<commit_message>
rever para eventual apresentação
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="48">
   <si>
     <t>projeto</t>
   </si>
@@ -92,21 +92,12 @@
     <t>pneus</t>
   </si>
   <si>
-    <t>Adequar o painel de DRE</t>
-  </si>
-  <si>
     <t>Criar indicadores e relatórios de pneus</t>
   </si>
   <si>
-    <t>Aguardando fim do projeto de melhoria de pneus</t>
-  </si>
-  <si>
     <t>Após o término da adequação da DRE</t>
   </si>
   <si>
-    <t>Entender e adequar indicadores do projeto TMS</t>
-  </si>
-  <si>
     <t>Performance de atendimento, movimentação de carga e outras informações relevantes para a operação de transporte.</t>
   </si>
   <si>
@@ -131,32 +122,59 @@
     <t>Relatórios</t>
   </si>
   <si>
-    <t>Soma</t>
-  </si>
-  <si>
-    <t>Média</t>
-  </si>
-  <si>
-    <t>Soma Acumulada</t>
-  </si>
-  <si>
-    <t>Contagem</t>
-  </si>
-  <si>
-    <t>Conforme demanda do setor pessoal</t>
-  </si>
-  <si>
     <t>Relatórios gerenciais</t>
   </si>
   <si>
     <t>Planilha de programação logística</t>
+  </si>
+  <si>
+    <t>Adequar a visão da DRE</t>
+  </si>
+  <si>
+    <t>Adequar a visão do balanço</t>
+  </si>
+  <si>
+    <t>Adequar indicadores do projeto TMS</t>
+  </si>
+  <si>
+    <t>Facilitar a análise da receita</t>
+  </si>
+  <si>
+    <t>Criar relatórios e indicadores da receita da operação de transporte.</t>
+  </si>
+  <si>
+    <t>Criar relatórios e indicadores para análise dos custos da operação de transporte.</t>
+  </si>
+  <si>
+    <t>Conforme demanda do setor pessoal.</t>
+  </si>
+  <si>
+    <t>Aguardando fim do projeto de melhoria de pneus.</t>
+  </si>
+  <si>
+    <t>A visão desejada por Porto e Cristianne não tem solução, após diversas tentativas e chamados abertos. O de número 14952058 foi o que mais se debruçou sobre a necessidade.</t>
+  </si>
+  <si>
+    <t>Após validação final com a logística, será necessário decidir onde se dará o acesso. Possivelmente no RM, com atualização manual, ou num projeto Fast Analytics separado, cuja carga se dará em curtos intervalos.</t>
+  </si>
+  <si>
+    <t>CRM</t>
+  </si>
+  <si>
+    <t>Adicionar o CRM ao painel de faturamento</t>
+  </si>
+  <si>
+    <t>Relatórios já criados, pendente validação pela Raquel, em reunião marcada para o dia 17/05.</t>
+  </si>
+  <si>
+    <t>Indicadores e relatórios</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -172,13 +190,51 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -193,7 +249,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -204,7 +260,19 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -487,7 +555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD11"/>
+  <dimension ref="A1:AD12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
@@ -495,33 +563,34 @@
     <col min="3" max="3" width="21.5703125" customWidth="1"/>
     <col min="4" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="112.5703125" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="119.140625" customWidth="1"/>
     <col min="29" max="29" width="25.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:30" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="8" t="s">
         <v>10</v>
       </c>
     </row>
@@ -533,7 +602,7 @@
         <v>9</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
@@ -543,7 +612,9 @@
       <c r="G2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="1"/>
+      <c r="H2" s="2" t="s">
+        <v>42</v>
+      </c>
       <c r="AC2" t="s">
         <v>5</v>
       </c>
@@ -551,14 +622,16 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:30" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C3" s="2"/>
+        <v>25</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>35</v>
+      </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
       <c r="F3" s="1" t="s">
@@ -567,8 +640,8 @@
       <c r="G3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>25</v>
+      <c r="H3" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="AC3" t="s">
         <v>6</v>
@@ -577,14 +650,16 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="2"/>
+        <v>26</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>37</v>
+      </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="F4" s="1" t="s">
@@ -593,7 +668,9 @@
       <c r="G4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="1"/>
+      <c r="H4" s="2" t="s">
+        <v>38</v>
+      </c>
       <c r="AC4" t="s">
         <v>7</v>
       </c>
@@ -602,11 +679,11 @@
       </c>
     </row>
     <row r="5" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="6" t="s">
         <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="3"/>
@@ -617,7 +694,9 @@
       <c r="G5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="1"/>
+      <c r="H5" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="AC5" t="s">
         <v>8</v>
       </c>
@@ -626,11 +705,11 @@
       </c>
     </row>
     <row r="6" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="6" t="s">
         <v>2</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="3"/>
@@ -641,17 +720,19 @@
       <c r="G6" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H6" s="1"/>
+      <c r="H6" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="AC6" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="6" t="s">
         <v>2</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="3"/>
@@ -662,20 +743,22 @@
       <c r="G7" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H7" s="1"/>
+      <c r="H7" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="AC7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:30" ht="45" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
+    <row r="8" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
         <v>2</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
@@ -685,16 +768,16 @@
       <c r="G8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H8" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="1:30" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="4" t="s">
+      <c r="H8" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>2</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="3"/>
@@ -705,17 +788,19 @@
       <c r="G9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H9" s="1"/>
+      <c r="H9" s="2" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="10" spans="1:30" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3">
@@ -727,19 +812,19 @@
       <c r="G10" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>24</v>
+      <c r="H10" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:30" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>33</v>
+      <c r="A11" s="7" t="s">
+        <v>30</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
@@ -749,16 +834,39 @@
       <c r="G11" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>39</v>
+      <c r="H11" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E12" s="3">
+        <v>45063</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F12">
       <formula1>$AC$3:$AC$7</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G11">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G12">
       <formula1>$AD$3:$AD$5</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
atualizações antes da visita do Porto 15/05/2023
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="49">
   <si>
     <t>projeto</t>
   </si>
@@ -137,9 +137,6 @@
     <t>Adequar indicadores do projeto TMS</t>
   </si>
   <si>
-    <t>Facilitar a análise da receita</t>
-  </si>
-  <si>
     <t>Criar relatórios e indicadores da receita da operação de transporte.</t>
   </si>
   <si>
@@ -152,12 +149,6 @@
     <t>Aguardando fim do projeto de melhoria de pneus.</t>
   </si>
   <si>
-    <t>A visão desejada por Porto e Cristianne não tem solução, após diversas tentativas e chamados abertos. O de número 14952058 foi o que mais se debruçou sobre a necessidade.</t>
-  </si>
-  <si>
-    <t>Após validação final com a logística, será necessário decidir onde se dará o acesso. Possivelmente no RM, com atualização manual, ou num projeto Fast Analytics separado, cuja carga se dará em curtos intervalos.</t>
-  </si>
-  <si>
     <t>CRM</t>
   </si>
   <si>
@@ -168,6 +159,18 @@
   </si>
   <si>
     <t>Indicadores e relatórios</t>
+  </si>
+  <si>
+    <t>Após validação final com a logística, será necessário decidir onde se dará o acesso. Possivelmente no RM, com atualização manual, ou num projeto Fast Analytics separado, o que viabilizaria uma carga em intervalos próximos à movimentação em tempo real.</t>
+  </si>
+  <si>
+    <t>A visão desejada por Porto e Cristianne não tem solução, após diversas tentativas e chamados abertos. O de número 14952058 foi o que mais se debruçou sobre a necessidade. Analisar as alternativas viáveis.</t>
+  </si>
+  <si>
+    <t>Facilitar a análise da receita da logística</t>
+  </si>
+  <si>
+    <t>MEMO</t>
   </si>
 </sst>
 </file>
@@ -555,7 +558,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AD12"/>
+  <dimension ref="A1:AE12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
@@ -564,11 +567,11 @@
     <col min="4" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="119.140625" customWidth="1"/>
-    <col min="29" max="29" width="25.5703125" customWidth="1"/>
+    <col min="8" max="9" width="119.140625" customWidth="1"/>
+    <col min="30" max="30" width="25.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -593,8 +596,11 @@
       <c r="H1" s="8" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+      <c r="I1" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -607,22 +613,23 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
       <c r="F2" s="1" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>14</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="AC2" t="s">
+        <v>46</v>
+      </c>
+      <c r="I2" s="2"/>
+      <c r="AD2" t="s">
         <v>5</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AE2" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
@@ -643,14 +650,15 @@
       <c r="H3" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="AC3" t="s">
+      <c r="I3" s="2"/>
+      <c r="AD3" t="s">
         <v>6</v>
       </c>
-      <c r="AD3" t="s">
+      <c r="AE3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>2</v>
       </c>
@@ -658,7 +666,7 @@
         <v>26</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -669,16 +677,17 @@
         <v>14</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="AC4" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" s="2"/>
+      <c r="AD4" t="s">
         <v>7</v>
       </c>
-      <c r="AD4" t="s">
+      <c r="AE4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>2</v>
       </c>
@@ -695,16 +704,17 @@
         <v>16</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" s="2"/>
+      <c r="AD5" t="s">
         <v>8</v>
       </c>
-      <c r="AD5" t="s">
+      <c r="AE5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>2</v>
       </c>
@@ -721,13 +731,14 @@
         <v>16</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC6" t="s">
+        <v>38</v>
+      </c>
+      <c r="I6" s="2"/>
+      <c r="AD6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:30" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>2</v>
       </c>
@@ -744,13 +755,14 @@
         <v>16</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="AC7" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" s="2"/>
+      <c r="AD7" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>2</v>
       </c>
@@ -771,8 +783,9 @@
       <c r="H8" s="2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="9" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+      <c r="I8" s="2"/>
+    </row>
+    <row r="9" spans="1:31" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>2</v>
       </c>
@@ -789,10 +802,11 @@
         <v>15</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="10" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="I9" s="2"/>
+    </row>
+    <row r="10" spans="1:31" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>3</v>
       </c>
@@ -813,10 +827,11 @@
         <v>16</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="11" spans="1:30" ht="15.75" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+      <c r="I10" s="2"/>
+    </row>
+    <row r="11" spans="1:31" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>30</v>
       </c>
@@ -829,24 +844,25 @@
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
       <c r="F11" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>15</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:30" ht="30" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+      <c r="I11" s="2"/>
+    </row>
+    <row r="12" spans="1:31" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>47</v>
-      </c>
       <c r="C12" s="2" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="E12" s="3">
         <v>45063</v>
@@ -858,16 +874,17 @@
         <v>15</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>46</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="I12" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F12">
-      <formula1>$AC$3:$AC$7</formula1>
+      <formula1>$AD$3:$AD$7</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G12">
-      <formula1>$AD$3:$AD$5</formula1>
+      <formula1>$AE$3:$AE$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
pedidos do Porto sobre o painel de DRE
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -164,13 +164,13 @@
     <t>Após validação final com a logística, será necessário decidir onde se dará o acesso. Possivelmente no RM, com atualização manual, ou num projeto Fast Analytics separado, o que viabilizaria uma carga em intervalos próximos à movimentação em tempo real.</t>
   </si>
   <si>
-    <t>A visão desejada por Porto e Cristianne não tem solução, após diversas tentativas e chamados abertos. O de número 14952058 foi o que mais se debruçou sobre a necessidade. Analisar as alternativas viáveis.</t>
-  </si>
-  <si>
     <t>Facilitar a análise da receita da logística</t>
   </si>
   <si>
     <t>MEMO</t>
+  </si>
+  <si>
+    <t>Porto sugeriu criar relatórios sem a AV, apenas com atual, mês do ano anterior, variação em valor e variação percentual. Assim também será possível criar relatórios com mais de um nível.</t>
   </si>
 </sst>
 </file>
@@ -202,7 +202,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -239,6 +239,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -252,7 +258,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -277,6 +283,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -597,7 +606,7 @@
         <v>10</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:31" ht="30" x14ac:dyDescent="0.25">
@@ -618,8 +627,8 @@
       <c r="G2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>46</v>
+      <c r="H2" s="9" t="s">
+        <v>48</v>
       </c>
       <c r="I2" s="2"/>
       <c r="AD2" t="s">
@@ -666,7 +675,7 @@
         <v>26</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>

</xml_diff>

<commit_message>
atualização pós reunião CRM 17/05/2023
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -155,9 +155,6 @@
     <t>Adicionar o CRM ao painel de faturamento</t>
   </si>
   <si>
-    <t>Relatórios já criados, pendente validação pela Raquel, em reunião marcada para o dia 17/05.</t>
-  </si>
-  <si>
     <t>Indicadores e relatórios</t>
   </si>
   <si>
@@ -170,7 +167,10 @@
     <t>MEMO</t>
   </si>
   <si>
-    <t>Porto sugeriu criar relatórios sem a AV, apenas com atual, mês do ano anterior, variação em valor e variação percentual. Assim também será possível criar relatórios com mais de um nível.</t>
+    <t>Porto sugeriu criar relatórios sem a AV, apenas com atual, mês do ano anterior, variação em valor e variação percentual. Assim também será possível criar relatórios com mais de um nível. Feito no dia 16/05/2023, aguardando validação e novas orientações.</t>
+  </si>
+  <si>
+    <t>Primeira visão aprovada. Para o dia 26/05/2023 a Raquel solicitou: quantidade de oportunidades ganhas e perdidas, e quantidades por vendedor. Silvio pediu um status simplificado, com oportunidades em aberto, perdidas e ganhas.</t>
   </si>
 </sst>
 </file>
@@ -202,7 +202,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -236,12 +236,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -284,7 +278,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -606,7 +600,7 @@
         <v>10</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:31" ht="30" x14ac:dyDescent="0.25">
@@ -628,7 +622,7 @@
         <v>14</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I2" s="2"/>
       <c r="AD2" t="s">
@@ -675,7 +669,7 @@
         <v>26</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -811,7 +805,7 @@
         <v>15</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="I9" s="2"/>
     </row>
@@ -868,7 +862,7 @@
         <v>41</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>42</v>
@@ -880,10 +874,10 @@
         <v>11</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="I12" s="2"/>
     </row>

</xml_diff>

<commit_message>
data fim CRM 26/05/2023
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -570,7 +570,8 @@
     <col min="4" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="119.140625" customWidth="1"/>
+    <col min="8" max="8" width="119.140625" customWidth="1"/>
+    <col min="9" max="9" width="119.140625" hidden="1" customWidth="1"/>
     <col min="30" max="30" width="25.5703125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -867,8 +868,11 @@
       <c r="C12" s="2" t="s">
         <v>42</v>
       </c>
+      <c r="D12" s="3">
+        <v>45036</v>
+      </c>
       <c r="E12" s="3">
-        <v>45063</v>
+        <v>45072</v>
       </c>
       <c r="F12" s="1" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
atualização status controladoria e RH
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -143,9 +143,6 @@
     <t>Criar relatórios e indicadores para análise dos custos da operação de transporte.</t>
   </si>
   <si>
-    <t>Conforme demanda do setor pessoal.</t>
-  </si>
-  <si>
     <t>Aguardando fim do projeto de melhoria de pneus.</t>
   </si>
   <si>
@@ -158,19 +155,22 @@
     <t>Indicadores e relatórios</t>
   </si>
   <si>
-    <t>Após validação final com a logística, será necessário decidir onde se dará o acesso. Possivelmente no RM, com atualização manual, ou num projeto Fast Analytics separado, o que viabilizaria uma carga em intervalos próximos à movimentação em tempo real.</t>
-  </si>
-  <si>
     <t>Facilitar a análise da receita da logística</t>
   </si>
   <si>
     <t>MEMO</t>
   </si>
   <si>
-    <t>Porto sugeriu criar relatórios sem a AV, apenas com atual, mês do ano anterior, variação em valor e variação percentual. Assim também será possível criar relatórios com mais de um nível. Feito no dia 16/05/2023, aguardando validação e novas orientações.</t>
-  </si>
-  <si>
     <t>Primeira visão aprovada. Para o dia 26/05/2023 a Raquel solicitou: quantidade de oportunidades ganhas e perdidas, e quantidades por vendedor. Silvio pediu um status simplificado, com oportunidades em aberto, perdidas e ganhas.</t>
+  </si>
+  <si>
+    <t>Conforme demanda do setor pessoal. No dia 24/05/2023 o relatório de VA, VT e cesta está sendo validado e alterado.</t>
+  </si>
+  <si>
+    <t>O projeto Fast Analytics não atenderia à necessidade, conforme análise do Paulino. Deixar para a Cristianne decidir se o RM satisfaz a demanda.</t>
+  </si>
+  <si>
+    <t>Em reunião no dia 22/05/2023 Porto decidiu deixar de lado a solução padrão do Fast Analytics para a controladoria.</t>
   </si>
 </sst>
 </file>
@@ -601,7 +601,7 @@
         <v>10</v>
       </c>
       <c r="I1" s="8" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:31" ht="30" x14ac:dyDescent="0.25">
@@ -620,10 +620,10 @@
         <v>11</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I2" s="2"/>
       <c r="AD2" t="s">
@@ -670,7 +670,7 @@
         <v>26</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="I9" s="2"/>
     </row>
@@ -831,7 +831,7 @@
         <v>16</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I10" s="2"/>
     </row>
@@ -854,19 +854,19 @@
         <v>15</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>39</v>
+        <v>46</v>
       </c>
       <c r="I11" s="2"/>
     </row>
     <row r="12" spans="1:31" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>41</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>42</v>
       </c>
       <c r="D12" s="3">
         <v>45036</v>
@@ -875,13 +875,13 @@
         <v>45072</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>16</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="I12" s="2"/>
     </row>

</xml_diff>

<commit_message>
solicitações do Silvio no painel DRE 25/05/2023
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -164,13 +164,13 @@
     <t>Primeira visão aprovada. Para o dia 26/05/2023 a Raquel solicitou: quantidade de oportunidades ganhas e perdidas, e quantidades por vendedor. Silvio pediu um status simplificado, com oportunidades em aberto, perdidas e ganhas.</t>
   </si>
   <si>
-    <t>Conforme demanda do setor pessoal. No dia 24/05/2023 o relatório de VA, VT e cesta está sendo validado e alterado.</t>
-  </si>
-  <si>
     <t>O projeto Fast Analytics não atenderia à necessidade, conforme análise do Paulino. Deixar para a Cristianne decidir se o RM satisfaz a demanda.</t>
   </si>
   <si>
-    <t>Em reunião no dia 22/05/2023 Porto decidiu deixar de lado a solução padrão do Fast Analytics para a controladoria.</t>
+    <t>Conforme demanda do setor pessoal. No dia 24/05/2023 o relatório de VA, VT e cesta está sendo validado e ajustado.</t>
+  </si>
+  <si>
+    <t>Em reunião no dia 22/05/2023 Porto decidiu deixar de lado a solução padrão do Fast Analytics para a controladoria. Em ligação com o Silvio no dia 25/05/2023, ele solicitou: relatórios separados de análise vertical e horizontal (por contas fixas) e alterar cores de variação % da DRE sintética, vendo variação por custo e despesa e receita.</t>
   </si>
 </sst>
 </file>
@@ -604,7 +604,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I9" s="2"/>
     </row>
@@ -854,7 +854,7 @@
         <v>15</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I11" s="2"/>
     </row>

</xml_diff>

<commit_message>
att pós reunião CRM
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -161,9 +161,6 @@
     <t>MEMO</t>
   </si>
   <si>
-    <t>Primeira visão aprovada. Para o dia 26/05/2023 a Raquel solicitou: quantidade de oportunidades ganhas e perdidas, e quantidades por vendedor. Silvio pediu um status simplificado, com oportunidades em aberto, perdidas e ganhas.</t>
-  </si>
-  <si>
     <t>O projeto Fast Analytics não atenderia à necessidade, conforme análise do Paulino. Deixar para a Cristianne decidir se o RM satisfaz a demanda.</t>
   </si>
   <si>
@@ -171,6 +168,9 @@
   </si>
   <si>
     <t>Em reunião no dia 22/05/2023 Porto decidiu deixar de lado a solução padrão do Fast Analytics para a controladoria. Em ligação com o Silvio no dia 25/05/2023, ele solicitou: relatórios separados de análise vertical e horizontal (por contas fixas) e alterar cores de variação % da DRE sintética, vendo variação por custo e despesa e receita.</t>
+  </si>
+  <si>
+    <t>Na reunião do dia 26/05/2023 a Raquel entendeu as informações de status e vendedor, e pediu para que este contivesse apenas os vendedores das oportunidades. Perguntou sobre a atividade e os produtos, e fica a pendência de incluir os itens da oportunidade, que são os serviços oferecidos. Incluir nos relatórios de oportunidades a quantidade e o percentual de ganhos, perdas etc.</t>
   </si>
 </sst>
 </file>
@@ -623,7 +623,7 @@
         <v>15</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I2" s="2"/>
       <c r="AD2" t="s">
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I9" s="2"/>
     </row>
@@ -854,11 +854,11 @@
         <v>15</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I11" s="2"/>
     </row>
-    <row r="12" spans="1:31" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:31" ht="60" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>40</v>
       </c>
@@ -881,7 +881,7 @@
         <v>16</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I12" s="2"/>
     </row>

</xml_diff>

<commit_message>
att status relatório cesta/VR/VT
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -164,13 +164,13 @@
     <t>O projeto Fast Analytics não atenderia à necessidade, conforme análise do Paulino. Deixar para a Cristianne decidir se o RM satisfaz a demanda.</t>
   </si>
   <si>
-    <t>Conforme demanda do setor pessoal. No dia 24/05/2023 o relatório de VA, VT e cesta está sendo validado e ajustado.</t>
-  </si>
-  <si>
     <t>Em reunião no dia 22/05/2023 Porto decidiu deixar de lado a solução padrão do Fast Analytics para a controladoria. Em ligação com o Silvio no dia 25/05/2023, ele solicitou: relatórios separados de análise vertical e horizontal (por contas fixas) e alterar cores de variação % da DRE sintética, vendo variação por custo e despesa e receita.</t>
   </si>
   <si>
     <t>Na reunião do dia 26/05/2023 a Raquel entendeu as informações de status e vendedor, e pediu para que este contivesse apenas os vendedores das oportunidades. Perguntou sobre a atividade e os produtos, e fica a pendência de incluir os itens da oportunidade, que são os serviços oferecidos. Incluir nos relatórios de oportunidades a quantidade e o percentual de ganhos, perdas etc.</t>
+  </si>
+  <si>
+    <t>Conforme demanda do setor pessoal. No dia 26/05/2023 apenas o relatório cesta não está correto.</t>
   </si>
 </sst>
 </file>
@@ -623,7 +623,7 @@
         <v>15</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I2" s="2"/>
       <c r="AD2" t="s">
@@ -854,7 +854,7 @@
         <v>15</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="I11" s="2"/>
     </row>
@@ -881,7 +881,7 @@
         <v>16</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I12" s="2"/>
     </row>

</xml_diff>

<commit_message>
att planilha de agendamentos TMS
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -161,9 +161,6 @@
     <t>MEMO</t>
   </si>
   <si>
-    <t>O projeto Fast Analytics não atenderia à necessidade, conforme análise do Paulino. Deixar para a Cristianne decidir se o RM satisfaz a demanda.</t>
-  </si>
-  <si>
     <t>Em reunião no dia 22/05/2023 Porto decidiu deixar de lado a solução padrão do Fast Analytics para a controladoria. Em ligação com o Silvio no dia 25/05/2023, ele solicitou: relatórios separados de análise vertical e horizontal (por contas fixas) e alterar cores de variação % da DRE sintética, vendo variação por custo e despesa e receita.</t>
   </si>
   <si>
@@ -171,6 +168,9 @@
   </si>
   <si>
     <t>Conforme demanda do setor pessoal. No dia 26/05/2023 apenas o relatório cesta não está correto.</t>
+  </si>
+  <si>
+    <t>O projeto Fast Analytics não atenderia à necessidade, conforme análise do Paulino. Deixar para a Cristianne decidir se o RM satisfaz a demanda. No dia 26/05/2023 a Cristianne sinalizou manter a planilha.</t>
   </si>
 </sst>
 </file>
@@ -623,7 +623,7 @@
         <v>15</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I2" s="2"/>
       <c r="AD2" t="s">
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="I9" s="2"/>
     </row>
@@ -854,7 +854,7 @@
         <v>15</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I11" s="2"/>
     </row>
@@ -881,7 +881,7 @@
         <v>16</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I12" s="2"/>
     </row>

</xml_diff>

<commit_message>
entrega do relatório de cesta, VT e VA
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -167,10 +167,10 @@
     <t>Na reunião do dia 26/05/2023 a Raquel entendeu as informações de status e vendedor, e pediu para que este contivesse apenas os vendedores das oportunidades. Perguntou sobre a atividade e os produtos, e fica a pendência de incluir os itens da oportunidade, que são os serviços oferecidos. Incluir nos relatórios de oportunidades a quantidade e o percentual de ganhos, perdas etc.</t>
   </si>
   <si>
-    <t>Conforme demanda do setor pessoal. No dia 26/05/2023 apenas o relatório cesta não está correto.</t>
-  </si>
-  <si>
     <t>O projeto Fast Analytics não atenderia à necessidade, conforme análise do Paulino. Deixar para a Cristianne decidir se o RM satisfaz a demanda. No dia 26/05/2023 a Cristianne sinalizou manter a planilha.</t>
+  </si>
+  <si>
+    <t>Conforme demanda do setor pessoal. No dia 29/05/2023 o relatório de cesta, VT e VA está entregue.</t>
   </si>
 </sst>
 </file>
@@ -806,7 +806,7 @@
         <v>15</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I9" s="2"/>
     </row>
@@ -854,7 +854,7 @@
         <v>15</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I11" s="2"/>
     </row>

</xml_diff>

<commit_message>
saldo atual de produtos e movimentações
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="52">
   <si>
     <t>projeto</t>
   </si>
@@ -164,13 +164,22 @@
     <t>Em reunião no dia 22/05/2023 Porto decidiu deixar de lado a solução padrão do Fast Analytics para a controladoria. Em ligação com o Silvio no dia 25/05/2023, ele solicitou: relatórios separados de análise vertical e horizontal (por contas fixas) e alterar cores de variação % da DRE sintética, vendo variação por custo e despesa e receita.</t>
   </si>
   <si>
-    <t>Na reunião do dia 26/05/2023 a Raquel entendeu as informações de status e vendedor, e pediu para que este contivesse apenas os vendedores das oportunidades. Perguntou sobre a atividade e os produtos, e fica a pendência de incluir os itens da oportunidade, que são os serviços oferecidos. Incluir nos relatórios de oportunidades a quantidade e o percentual de ganhos, perdas etc.</t>
-  </si>
-  <si>
     <t>O projeto Fast Analytics não atenderia à necessidade, conforme análise do Paulino. Deixar para a Cristianne decidir se o RM satisfaz a demanda. No dia 26/05/2023 a Cristianne sinalizou manter a planilha.</t>
   </si>
   <si>
     <t>Conforme demanda do setor pessoal. No dia 29/05/2023 o relatório de cesta, VT e VA está entregue.</t>
+  </si>
+  <si>
+    <t>Painéis de gestão de manutenção</t>
+  </si>
+  <si>
+    <t>Relatórios, gráficos e indicadores dos sistemas de manutenção</t>
+  </si>
+  <si>
+    <t>Em email no dia 07/06/2023, a Raquel pediu para verificar a quantidade, divergente, de oportunidades por cliente e por prospect.</t>
+  </si>
+  <si>
+    <t>Alterações conforme solicitações do Silvio, e de outras necessidades. Incluir gráfico de MDO e de terceiros no painel Frota &gt; Manutenção.</t>
   </si>
 </sst>
 </file>
@@ -561,7 +570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AE12"/>
+  <dimension ref="A1:AE13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
@@ -806,7 +815,7 @@
         <v>15</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="I9" s="2"/>
     </row>
@@ -835,62 +844,85 @@
       </c>
       <c r="I10" s="2"/>
     </row>
-    <row r="11" spans="1:31" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
-        <v>30</v>
+    <row r="11" spans="1:31" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>3</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>32</v>
+        <v>49</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
       <c r="F11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I11" s="2"/>
+    </row>
+    <row r="12" spans="1:31" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G12" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H11" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="I11" s="2"/>
-    </row>
-    <row r="12" spans="1:31" ht="60" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+      <c r="H12" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="I12" s="2"/>
+    </row>
+    <row r="13" spans="1:31" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D13" s="3">
         <v>45036</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E13" s="3">
         <v>45072</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="G13" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="H12" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I12" s="2"/>
+      <c r="H13" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="I13" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F12">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F13">
       <formula1>$AD$3:$AD$7</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G12">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G13">
       <formula1>$AE$3:$AE$5</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
sem data ini e fim
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="50">
   <si>
     <t>projeto</t>
   </si>
@@ -78,12 +78,6 @@
   </si>
   <si>
     <t>descrição</t>
-  </si>
-  <si>
-    <t>início</t>
-  </si>
-  <si>
-    <t>fim</t>
   </si>
   <si>
     <t>indicadores logística</t>
@@ -261,16 +255,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -570,360 +561,323 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AE13"/>
+  <dimension ref="A1:AC13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
     <col min="2" max="2" width="31" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.5703125" customWidth="1"/>
-    <col min="4" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="119.140625" customWidth="1"/>
-    <col min="9" max="9" width="119.140625" hidden="1" customWidth="1"/>
-    <col min="30" max="30" width="25.5703125" customWidth="1"/>
+    <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="119.140625" customWidth="1"/>
+    <col min="7" max="7" width="119.140625" hidden="1" customWidth="1"/>
+    <col min="28" max="28" width="25.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:29" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="F1" s="8" t="s">
+      <c r="D1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="E1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="F1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="8" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="2" spans="1:31" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="G1" s="7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" s="2"/>
+      <c r="AB2" t="s">
+        <v>5</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="AB3" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="AB4" t="s">
+        <v>7</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="AB5" t="s">
+        <v>8</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" s="2"/>
+      <c r="AB6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="2"/>
+      <c r="D7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" s="2"/>
+      <c r="AB7" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="1" t="s">
+      <c r="D8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G8" s="2"/>
+    </row>
+    <row r="9" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="2"/>
+      <c r="D9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="9" t="s">
+      <c r="F9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="G9" s="2"/>
+    </row>
+    <row r="10" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" s="2"/>
+    </row>
+    <row r="11" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="G11" s="2"/>
+    </row>
+    <row r="12" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="I2" s="2"/>
-      <c r="AD2" t="s">
-        <v>5</v>
-      </c>
-      <c r="AE2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:31" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I3" s="2"/>
-      <c r="AD3" t="s">
-        <v>6</v>
-      </c>
-      <c r="AE3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:31" ht="30" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="1" t="s">
+      <c r="G12" s="2"/>
+    </row>
+    <row r="13" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="I4" s="2"/>
-      <c r="AD4" t="s">
-        <v>7</v>
-      </c>
-      <c r="AE4" t="s">
+      <c r="E13" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I5" s="2"/>
-      <c r="AD5" t="s">
-        <v>8</v>
-      </c>
-      <c r="AE5" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I6" s="2"/>
-      <c r="AD6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:31" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I7" s="2"/>
-      <c r="AD7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:31" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="I8" s="2"/>
-    </row>
-    <row r="9" spans="1:31" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="I9" s="2"/>
-    </row>
-    <row r="10" spans="1:31" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3">
-        <v>45137</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="I10" s="2"/>
-    </row>
-    <row r="11" spans="1:31" ht="60" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="1" t="s">
+      <c r="F13" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H11" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="I11" s="2"/>
-    </row>
-    <row r="12" spans="1:31" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="I12" s="2"/>
-    </row>
-    <row r="13" spans="1:31" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D13" s="3">
-        <v>45036</v>
-      </c>
-      <c r="E13" s="3">
-        <v>45072</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="I13" s="2"/>
+      <c r="G13" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F2:F13">
-      <formula1>$AD$3:$AD$7</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D13">
+      <formula1>$AB$3:$AB$7</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G2:G13">
-      <formula1>$AE$3:$AE$5</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E13">
+      <formula1>$AC$3:$AC$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
att DRE, TMS, CRM, MNT
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -14,6 +14,9 @@
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Plan1!$A$1:$G$14</definedName>
+  </definedNames>
   <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -24,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="54">
   <si>
     <t>projeto</t>
   </si>
@@ -119,9 +122,6 @@
     <t>Relatórios gerenciais</t>
   </si>
   <si>
-    <t>Planilha de programação logística</t>
-  </si>
-  <si>
     <t>Adequar a visão da DRE</t>
   </si>
   <si>
@@ -155,18 +155,12 @@
     <t>MEMO</t>
   </si>
   <si>
-    <t>Em reunião no dia 22/05/2023 Porto decidiu deixar de lado a solução padrão do Fast Analytics para a controladoria. Em ligação com o Silvio no dia 25/05/2023, ele solicitou: relatórios separados de análise vertical e horizontal (por contas fixas) e alterar cores de variação % da DRE sintética, vendo variação por custo e despesa e receita.</t>
-  </si>
-  <si>
     <t>O projeto Fast Analytics não atenderia à necessidade, conforme análise do Paulino. Deixar para a Cristianne decidir se o RM satisfaz a demanda. No dia 26/05/2023 a Cristianne sinalizou manter a planilha.</t>
   </si>
   <si>
     <t>Conforme demanda do setor pessoal. No dia 29/05/2023 o relatório de cesta, VT e VA está entregue.</t>
   </si>
   <si>
-    <t>Painéis de gestão de manutenção</t>
-  </si>
-  <si>
     <t>Relatórios, gráficos e indicadores dos sistemas de manutenção</t>
   </si>
   <si>
@@ -174,6 +168,27 @@
   </si>
   <si>
     <t>Alterações conforme solicitações do Silvio, e de outras necessidades. Incluir gráfico de MDO e de terceiros no painel Frota &gt; Manutenção.</t>
+  </si>
+  <si>
+    <t>Energia do Bardella</t>
+  </si>
+  <si>
+    <t>Painéis</t>
+  </si>
+  <si>
+    <t>Planilha logística</t>
+  </si>
+  <si>
+    <t>Criar controle de consumo de energia e do contador do Bardella</t>
+  </si>
+  <si>
+    <t>A partir da NF recebida mensalmente é possível registrar o abastecimento de energia, com kWh, valor, horímetro e horas rodadas.</t>
+  </si>
+  <si>
+    <t>Em ligação com o Silvio no dia 25/05/2023, ele solicitou: relatórios separados de análise vertical e horizontal (por contas fixas) e alterar cores de variação % da DRE sintética, vendo variação por custo e despesa e receita. No dia 12/06/2023 o Porto pediu a criação de um projeto para levar a DRE para o RM.</t>
+  </si>
+  <si>
+    <t>Possibilitar a análise dos custos da logística</t>
   </si>
 </sst>
 </file>
@@ -561,12 +576,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AC13"/>
+  <dimension ref="A1:AC14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
-    <col min="2" max="2" width="31" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.5703125" customWidth="1"/>
+    <col min="2" max="2" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.28515625" customWidth="1"/>
     <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="119.140625" customWidth="1"/>
@@ -594,7 +609,7 @@
         <v>10</v>
       </c>
       <c r="G1" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:29" ht="45" x14ac:dyDescent="0.25">
@@ -605,16 +620,16 @@
         <v>9</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>43</v>
+        <v>52</v>
       </c>
       <c r="G2" s="2"/>
       <c r="AB2" t="s">
@@ -632,7 +647,7 @@
         <v>23</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>12</v>
@@ -659,7 +674,7 @@
         <v>24</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>8</v>
@@ -668,7 +683,7 @@
         <v>14</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G4" s="2"/>
       <c r="AB4" t="s">
@@ -685,7 +700,9 @@
       <c r="B5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="2"/>
+      <c r="C5" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="D5" s="1" t="s">
         <v>8</v>
       </c>
@@ -693,7 +710,7 @@
         <v>16</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G5" s="2"/>
       <c r="AB5" t="s">
@@ -710,7 +727,9 @@
       <c r="B6" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="2"/>
+      <c r="C6" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="D6" s="1" t="s">
         <v>8</v>
       </c>
@@ -718,7 +737,7 @@
         <v>16</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G6" s="2"/>
       <c r="AB6" t="s">
@@ -732,7 +751,9 @@
       <c r="B7" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="2"/>
+      <c r="C7" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="D7" s="1" t="s">
         <v>12</v>
       </c>
@@ -740,7 +761,7 @@
         <v>16</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G7" s="2"/>
       <c r="AB7" t="s">
@@ -755,7 +776,7 @@
         <v>18</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>6</v>
@@ -773,17 +794,17 @@
         <v>2</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>15</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G9" s="2"/>
     </row>
@@ -804,7 +825,7 @@
         <v>16</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G10" s="2"/>
     </row>
@@ -813,10 +834,10 @@
         <v>3</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>6</v>
@@ -825,58 +846,79 @@
         <v>14</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="G11" s="2"/>
     </row>
-    <row r="12" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="6" t="s">
+    <row r="12" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="G12" s="2"/>
+    </row>
+    <row r="13" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B13" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D13" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E13" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F13" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" s="2"/>
+    </row>
+    <row r="14" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G12" s="2"/>
-    </row>
-    <row r="13" spans="1:29" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="G13" s="2"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G14"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D13">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D14">
       <formula1>$AB$3:$AB$7</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E13">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E14">
       <formula1>$AC$3:$AC$5</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
DRE pronta para apresentação
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -185,10 +185,10 @@
     <t>A partir da NF recebida mensalmente é possível registrar o abastecimento de energia, com kWh, valor, horímetro e horas rodadas.</t>
   </si>
   <si>
-    <t>Em ligação com o Silvio no dia 25/05/2023, ele solicitou: relatórios separados de análise vertical e horizontal (por contas fixas) e alterar cores de variação % da DRE sintética, vendo variação por custo e despesa e receita. No dia 12/06/2023 o Porto pediu a criação de um projeto para levar a DRE para o RM.</t>
-  </si>
-  <si>
     <t>Possibilitar a análise dos custos da logística</t>
+  </si>
+  <si>
+    <t>Em ligação com o Silvio no dia 25/05/2023, ele solicitou: relatórios separados de análise vertical e horizontal (por contas fixas) e alterar cores de variação % da DRE sintética, vendo variação por custo e despesa e receita. No dia 12/06/2023 o Porto pediu a criação de um projeto para levar a DRE para o RM. Em reunião no dia 19/06/2023 o Porto e Cristianne informaram que os valores estavam corretos, e que bastaria ajustar ligeiramente os relatórios.</t>
   </si>
 </sst>
 </file>
@@ -612,7 +612,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -629,7 +629,7 @@
         <v>14</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G2" s="2"/>
       <c r="AB2" t="s">
@@ -701,7 +701,7 @@
         <v>25</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>8</v>
@@ -728,7 +728,7 @@
         <v>26</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>8</v>
@@ -752,7 +752,7 @@
         <v>27</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
att status DRE e OBS do contador do bardella
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="55">
   <si>
     <t>projeto</t>
   </si>
@@ -182,13 +182,16 @@
     <t>Criar controle de consumo de energia e do contador do Bardella</t>
   </si>
   <si>
-    <t>A partir da NF recebida mensalmente é possível registrar o abastecimento de energia, com kWh, valor, horímetro e horas rodadas.</t>
-  </si>
-  <si>
     <t>Possibilitar a análise dos custos da logística</t>
   </si>
   <si>
-    <t>Em ligação com o Silvio no dia 25/05/2023, ele solicitou: relatórios separados de análise vertical e horizontal (por contas fixas) e alterar cores de variação % da DRE sintética, vendo variação por custo e despesa e receita. No dia 12/06/2023 o Porto pediu a criação de um projeto para levar a DRE para o RM. Em reunião no dia 19/06/2023 o Porto e Cristianne informaram que os valores estavam corretos, e que bastaria ajustar ligeiramente os relatórios.</t>
+    <t>Em ligação com o Silvio no dia 25/05/2023, ele solicitou: relatórios separados de análise vertical e horizontal (por contas fixas) e alterar cores de variação % da DRE sintética, vendo variação por custo e despesa e receita. No dia 12/06/2023 o Porto pediu a criação de um projeto para levar a DRE para o RM. Em reunião no dia 19/06/2023 o Porto e Cristianne informaram que os valores estavam corretos, e que bastaria ajustar ligeiramente os relatórios. No dia 20/06/2023 a Cristianne validou o painel de DRE.</t>
+  </si>
+  <si>
+    <t>A partir da NF recebida mensalmente é possível registrar o abastecimento de energia, com kWh, valor, horímetro e horas rodadas. Criar produto energia elétrica do Bardella, posto, vincular combustível ao produto e testar a movimentação.</t>
+  </si>
+  <si>
+    <t>Automatizar informações manuais da planilha</t>
   </si>
 </sst>
 </file>
@@ -582,8 +585,8 @@
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
     <col min="2" max="2" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31.28515625" customWidth="1"/>
-    <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="119.140625" customWidth="1"/>
     <col min="7" max="7" width="119.140625" hidden="1" customWidth="1"/>
     <col min="28" max="28" width="25.5703125" customWidth="1"/>
@@ -629,7 +632,7 @@
         <v>14</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G2" s="2"/>
       <c r="AB2" t="s">
@@ -701,7 +704,7 @@
         <v>25</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>8</v>
@@ -728,7 +731,7 @@
         <v>26</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>8</v>
@@ -752,7 +755,7 @@
         <v>27</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>12</v>
@@ -796,7 +799,9 @@
       <c r="B9" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="2"/>
+      <c r="C9" s="2" t="s">
+        <v>54</v>
+      </c>
       <c r="D9" s="1" t="s">
         <v>7</v>
       </c>
@@ -867,7 +872,7 @@
         <v>14</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G12" s="2"/>
     </row>

</xml_diff>

<commit_message>
alterações solicitadas pelo Silvio aos 26 e 27
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -167,9 +167,6 @@
     <t>Em email no dia 07/06/2023, a Raquel pediu para verificar a quantidade, divergente, de oportunidades por cliente e por prospect.</t>
   </si>
   <si>
-    <t>Alterações conforme solicitações do Silvio, e de outras necessidades. Incluir gráfico de MDO e de terceiros no painel Frota &gt; Manutenção.</t>
-  </si>
-  <si>
     <t>Energia do Bardella</t>
   </si>
   <si>
@@ -192,6 +189,9 @@
   </si>
   <si>
     <t>Automatizar informações manuais da planilha</t>
+  </si>
+  <si>
+    <t>Alterações conforme solicitações do Silvio, e de outras necessidades. Incluir gráfico de MDO e de terceiros no painel Frota &gt; Manutenção. Após reuniões nos dias 26 e 27 de junho, alterar gráficos de manutenção e combustível, a fim de separar aqueles com km daqueles com hora, além de solicitações conforme informado por Wellington no dia 27/06/2023.</t>
   </si>
 </sst>
 </file>
@@ -632,7 +632,7 @@
         <v>14</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G2" s="2"/>
       <c r="AB2" t="s">
@@ -704,7 +704,7 @@
         <v>25</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>8</v>
@@ -731,7 +731,7 @@
         <v>26</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>8</v>
@@ -755,7 +755,7 @@
         <v>27</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>12</v>
@@ -797,10 +797,10 @@
         <v>2</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>7</v>
@@ -834,12 +834,12 @@
       </c>
       <c r="G10" s="2"/>
     </row>
-    <row r="11" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>3</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>44</v>
@@ -851,7 +851,7 @@
         <v>14</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="G11" s="2"/>
     </row>
@@ -860,10 +860,10 @@
         <v>3</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>12</v>
@@ -872,7 +872,7 @@
         <v>14</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G12" s="2"/>
     </row>

</xml_diff>

<commit_message>
envio para o Silvio e cc em 29/06/2023
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="68">
   <si>
     <t>projeto</t>
   </si>
@@ -50,9 +50,6 @@
     <t>em andamento</t>
   </si>
   <si>
-    <t>atrasado</t>
-  </si>
-  <si>
     <t>DRE</t>
   </si>
   <si>
@@ -80,12 +77,6 @@
     <t>descrição</t>
   </si>
   <si>
-    <t>indicadores logística</t>
-  </si>
-  <si>
-    <t>pneus</t>
-  </si>
-  <si>
     <t>Criar indicadores e relatórios de pneus</t>
   </si>
   <si>
@@ -134,9 +125,6 @@
     <t>Adicionar o CRM ao painel de faturamento</t>
   </si>
   <si>
-    <t>Indicadores e relatórios</t>
-  </si>
-  <si>
     <t>Facilitar a análise da receita da logística</t>
   </si>
   <si>
@@ -146,9 +134,6 @@
     <t>Relatórios, gráficos e indicadores dos sistemas de manutenção</t>
   </si>
   <si>
-    <t>Em email no dia 07/06/2023, a Raquel pediu para verificar a quantidade, divergente, de oportunidades por cliente e por prospect.</t>
-  </si>
-  <si>
     <t>Energia do Bardella</t>
   </si>
   <si>
@@ -170,9 +155,6 @@
     <t>A partir da NF recebida mensalmente é possível registrar o abastecimento de energia, com kWh, valor, horímetro e horas rodadas. Criar posto e produto energia elétrica do Bardella, vincular tipo de combustível (energia) ao produto, testar a movimentação e o cálculo da média.</t>
   </si>
   <si>
-    <t>O projeto Fast Analytics não atenderia à necessidade, conforme análise do Paulino. No dia 26/05/2023 a Cristianne sinalizou também manter a planilha, já que sua substituição não seria viável nem pelo RM, após análise das duas soluções.</t>
-  </si>
-  <si>
     <t>em pausa</t>
   </si>
   <si>
@@ -206,31 +188,49 @@
     <t>Compras</t>
   </si>
   <si>
-    <t>Relatórios de compras</t>
-  </si>
-  <si>
     <t>Conforme demanda do setor pessoal.</t>
   </si>
   <si>
     <t>Visto que o relatório EIR não é integrado à rotina de OS portuária, não é possível relacionar quais contêineres foram devolvidos por quais motoristas, apesar do registro do serviço prestado de devolução de contêiner vazio, pela rotina de OS portuária no faturamento. Sugestão de alterar a customização para incluir um campo com a informação do motorista que fez a devolução.</t>
   </si>
   <si>
-    <t>Alterações conforme solicitações do Silvio, e de outras necessidades, como criar gráficos para a reunião mensal de indicadores. Incluir gráfico de MDO e de terceiros no painel Frota &gt; Manutenção. Após reuniões nos dias 26 e 27 de junho, alterar gráficos de manutenção e combustível, a fim de separar aqueles com km daqueles com hora, além de solicitações conforme informado por Wellington no dia 27/06/2023.</t>
-  </si>
-  <si>
     <t>Automatizar carga de dados não controlados pelo sistema</t>
   </si>
   <si>
-    <t>Conforme solicitado pelo Wellington em reunião no dia 24/06/2023, criar um método de carga automática dos dados de disponibilidade, veículos aguardando peças e em serviços externos, que hoje são informações manualmente preenchidas para a reunião mensal. Projeto de criação de planilha preenchida pelo setor de manutenção com um leiaute específico para a carga junto das demais informações do setor, como OS realizadas e abastecimentos.</t>
-  </si>
-  <si>
-    <t>Conforme demanda do Manoel Junior, os relatórios são criados junto à Fátima.</t>
-  </si>
-  <si>
-    <t>Em ligação com o Silvio no dia 25/05/2023, solicitou: relatórios separados de análise vertical e horizontal (por contas fixas). No dia 12/06/2023 o Porto pediu a criação de um projeto para levar a DRE para o RM. Em reunião no dia 19/06/2023, Porto e Cristianne informaram que os valores estavam corretos, e que bastaria ajustar ligeiramente os relatórios, ajustes que foram confirmados pela Cristianne no dia 20/06/2023, dia em que deu aval para utilização do painel.</t>
-  </si>
-  <si>
     <t>Criar relatórios e indicadores da receita da operação de transporte. Necessário modelar a obtenção das receitas extras das viagens, como aquelas de RPS e nota de débito, e criar relatórios que confirmem essas informações ou não.</t>
+  </si>
+  <si>
+    <t>O projeto Fast Analytics não atenderia à necessidade, conforme análise do Paulino. Cristianne também sinalizou manter a planilha, já que sua substituição não seria viável nem pelo RM, após análise das duas soluções.</t>
+  </si>
+  <si>
+    <t>Incluir gráfico de MDO e de terceiros no painel Frota &gt; Manutenção. Após reuniões com Silvio, Porto e Cristianne, alterar gráficos de manutenção e combustível, a fim de separar aqueles com km daqueles com hora. Outras solicitações conforme informado por Wellington por email.</t>
+  </si>
+  <si>
+    <t>Conforme solicitado pelo Wellington em reunião quinzenal, criar um método de carga automática dos dados de disponibilidade, veículos aguardando peças e em serviços externos, que hoje são informações manualmente preenchidas para a reunião mensal. Projeto de criação de planilha preenchida pelo setor de manutenção com um leiaute específico para a carga junto das demais informações do setor, como OS realizadas e abastecimentos.</t>
+  </si>
+  <si>
+    <t>Raquel pediu para verificar a quantidade, divergente, de oportunidades por cliente e por prospect, no projeto já apresentado de indicadores do sistema de CRM.</t>
+  </si>
+  <si>
+    <t>indicadores</t>
+  </si>
+  <si>
+    <t>Pneus</t>
+  </si>
+  <si>
+    <t>Custos</t>
+  </si>
+  <si>
+    <t>Otimizar a análise do custo da operação portuária</t>
+  </si>
+  <si>
+    <t>Os custos são apropriados de acordo com rotina customizada no módulo de faturamento. A validação e a análise dos valores, pela contabilidade, apoia-se em relatórios existentes ou criados com essa finalidade, e são disponibilizados nos cubos do RM.</t>
+  </si>
+  <si>
+    <t>Criar relatórios separados de análise vertical e horizontal (por contas fixas), após solicitação do Silvio. Porto pediu a criação de um projeto para levar a DRE para o RM. Em reunião, Porto e Cristianne informaram que os valores estavam corretos, e que bastaria ajustar ligeiramente os relatórios, ajustes que foram confirmados pela Cristianne, assim como a utilização do painel a partir de então.</t>
+  </si>
+  <si>
+    <t>Conforme demanda do Manoel Junior, os relatórios são criados ou emitidos junto com a Fátima.</t>
   </si>
 </sst>
 </file>
@@ -285,7 +285,7 @@
       <scheme val="major"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -349,6 +349,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -374,7 +386,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -438,6 +450,18 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -719,13 +743,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AC17"/>
+  <dimension ref="A1:AC18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
     <col min="2" max="2" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38.7109375" customWidth="1"/>
-    <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="119.140625" customWidth="1"/>
     <col min="7" max="7" width="119.140625" hidden="1" customWidth="1"/>
@@ -740,36 +764,36 @@
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F2" s="18" t="s">
         <v>66</v>
@@ -779,7 +803,7 @@
         <v>5</v>
       </c>
       <c r="AC2" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:29" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -787,175 +811,172 @@
         <v>1</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="G3" s="1"/>
       <c r="AB3" s="5" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AC3" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="19" t="s">
-        <v>67</v>
+      <c r="B4" s="25" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F4" s="24" t="s">
+        <v>56</v>
       </c>
       <c r="G4" s="1"/>
       <c r="AB4" s="5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AC4" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:29" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="F5" s="19" t="s">
-        <v>31</v>
+      <c r="B5" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F5" s="24" t="s">
+        <v>28</v>
       </c>
       <c r="G5" s="1"/>
       <c r="AB5" s="5" t="s">
-        <v>6</v>
+        <v>42</v>
       </c>
       <c r="AC5" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" s="23" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="1:29" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" s="19" t="s">
-        <v>55</v>
+      <c r="F6" s="24" t="s">
+        <v>49</v>
       </c>
       <c r="G6" s="1"/>
       <c r="AB6" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="AC6" s="5"/>
     </row>
     <row r="7" spans="1:29" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="19" t="s">
-        <v>56</v>
+      <c r="B7" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" s="24" t="s">
+        <v>50</v>
       </c>
       <c r="G7" s="1"/>
-      <c r="AB7" s="5" t="s">
-        <v>50</v>
+      <c r="AB7" s="6" t="s">
+        <v>43</v>
       </c>
       <c r="AC7" s="5"/>
     </row>
     <row r="8" spans="1:29" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" s="15" t="s">
+      <c r="B8" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="24" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="E8" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="F8" s="19" t="s">
+      <c r="E8" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" s="1"/>
+      <c r="AC8" s="6"/>
+    </row>
+    <row r="9" spans="1:29" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="24" t="s">
         <v>57</v>
-      </c>
-      <c r="G8" s="1"/>
-      <c r="AB8" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="AC8" s="6"/>
-    </row>
-    <row r="9" spans="1:29" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="E9" s="15" t="s">
-        <v>14</v>
-      </c>
-      <c r="F9" s="19" t="s">
-        <v>47</v>
       </c>
       <c r="G9" s="1"/>
     </row>
@@ -964,163 +985,183 @@
         <v>3</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>18</v>
+        <v>62</v>
       </c>
       <c r="C10" s="20" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="E10" s="16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F10" s="20" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:29" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29" ht="57" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>3</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D11" s="16" t="s">
         <v>6</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="G11" s="1"/>
     </row>
-    <row r="12" spans="1:29" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:29" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>3</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="D12" s="16" t="s">
         <v>6</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="G12" s="1"/>
     </row>
-    <row r="13" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:29" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>3</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="C13" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="16" t="s">
-        <v>49</v>
-      </c>
       <c r="E13" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="G13" s="1"/>
+    </row>
+    <row r="14" spans="1:29" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="F13" s="20" t="s">
-        <v>46</v>
-      </c>
-      <c r="G13" s="1"/>
-    </row>
-    <row r="14" spans="1:29" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>26</v>
-      </c>
-      <c r="C14" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="E14" s="17" t="s">
+      <c r="F14" s="19" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="F14" s="21" t="s">
+      <c r="F15" s="19" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:29" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="21" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="21" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="F17" s="21" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="C15" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="E15" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="F15" s="21" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="16" spans="1:29" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="B16" s="12" t="s">
+    <row r="18" spans="1:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="C16" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="D16" s="17" t="s">
-        <v>49</v>
-      </c>
-      <c r="E16" s="17" t="s">
+      <c r="B18" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="F16" s="21" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="C17" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="D17" s="17" t="s">
-        <v>50</v>
-      </c>
-      <c r="E17" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="F17" s="21" t="s">
-        <v>65</v>
+      <c r="F18" s="21" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1129,11 +1170,11 @@
     <sortCondition ref="AB3"/>
   </sortState>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D17">
-      <formula1>$AB$3:$AB$10</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E18">
+      <formula1>$AC$3:$AC$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E17">
-      <formula1>$AC$3:$AC$5</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D18">
+      <formula1>$AB$3:$AB$9</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
ajustes Silvio painel manutenção
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -230,7 +230,7 @@
     <t>Paulo Cesar está conferindo os valores e, ao mesmo tempo, solicitando verificações dos dados, para que o painel esteja compatível com os relatórios do sistema. Balancete até então ok, mas necessário ajustar o leiaute, e corrigir o balanço.</t>
   </si>
   <si>
-    <t>Incluir gráfico de MDO e de terceiros no painel Frota &gt; Manutenção. Gráficos de manutenção e combustível agora exibem apenas km ou apenas hora.</t>
+    <t>Incluir gráfico de MDO e de terceiros no painel Frota &gt; Manutenção. Alterar gráfico acumulado da aba "anual".</t>
   </si>
 </sst>
 </file>
@@ -1037,7 +1037,7 @@
         <v>53</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="E12" s="16" t="s">
         <v>12</v>
@@ -1058,7 +1058,7 @@
         <v>38</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="E13" s="16" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
add linha com o custo TMS em planilha
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="71">
   <si>
     <t>projeto</t>
   </si>
@@ -231,6 +231,15 @@
   </si>
   <si>
     <t>Paulo Cesar está conferindo os valores e, ao mesmo tempo, solicitando verificações dos dados, para que o painel esteja compatível com os relatórios do sistema. Balancete até então ok, mas necessário ajustar o leiaute, e corrigir o balanço. Verificar total da conta sintética, adicionar valor de "saldo inicial do ano". Relatório de balanço por ano atual e ano anterior.</t>
+  </si>
+  <si>
+    <t>Custo em planilha</t>
+  </si>
+  <si>
+    <t>Conforme demanda do analista de custos (Paulo Cesar) por relatórios por ele compilados para criar o custo do TMS em Excel.</t>
+  </si>
+  <si>
+    <t>Criar e emitir relatórios dos custos</t>
   </si>
 </sst>
 </file>
@@ -744,7 +753,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AC18"/>
+  <dimension ref="A1:AC19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
@@ -946,19 +955,19 @@
         <v>2</v>
       </c>
       <c r="B8" s="25" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>27</v>
+        <v>70</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="G8" s="1"/>
       <c r="AC8" s="6"/>
@@ -968,61 +977,61 @@
         <v>2</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>37</v>
+        <v>57</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>40</v>
+        <v>27</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E9" s="23" t="s">
         <v>13</v>
       </c>
       <c r="F9" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="1:29" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="G9" s="1"/>
-    </row>
-    <row r="10" spans="1:29" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C10" s="20" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="F10" s="20" t="s">
-        <v>29</v>
-      </c>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>3</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>66</v>
+        <v>29</v>
       </c>
       <c r="G11" s="1"/>
     </row>
@@ -1034,16 +1043,16 @@
         <v>36</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="E12" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>56</v>
+        <v>66</v>
       </c>
       <c r="G12" s="1"/>
     </row>
@@ -1051,43 +1060,43 @@
       <c r="A13" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="B13" s="13" t="s">
-        <v>35</v>
+      <c r="B13" s="3" t="s">
+        <v>36</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>38</v>
+        <v>53</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="E13" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="G13" s="1"/>
       <c r="J13" s="26"/>
       <c r="L13" s="26"/>
     </row>
     <row r="14" spans="1:29" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>47</v>
-      </c>
-      <c r="D14" s="15" t="s">
+      <c r="A14" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="C14" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="F14" s="19" t="s">
-        <v>65</v>
+      <c r="E14" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="20" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1095,50 +1104,50 @@
         <v>45</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>59</v>
+        <v>46</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>60</v>
+        <v>47</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>9</v>
       </c>
       <c r="E15" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="19" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="16" spans="1:29" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="F15" s="19" t="s">
+      <c r="F16" s="19" t="s">
         <v>61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:29" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="C16" s="21" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="E16" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" s="21" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>36</v>
+        <v>23</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="D17" s="17" t="s">
         <v>44</v>
@@ -1147,26 +1156,46 @@
         <v>13</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
-        <v>51</v>
+        <v>30</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="D18" s="17" t="s">
         <v>44</v>
       </c>
       <c r="E18" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="21" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="F18" s="21" t="s">
+      <c r="F19" s="21" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1176,10 +1205,10 @@
     <sortCondition ref="AB3"/>
   </sortState>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E18">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E19">
       <formula1>$AC$3:$AC$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D18">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D19">
       <formula1>$AB$3:$AB$9</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
att controladoria; balanço e balancete
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -230,9 +230,6 @@
     <t>Incluir gráfico de MDO e de terceiros no painel Frota &gt; Manutenção. Alterar gráfico acumulado da aba "anual".</t>
   </si>
   <si>
-    <t>Paulo Cesar está conferindo os valores e, ao mesmo tempo, solicitando verificações dos dados, para que o painel esteja compatível com os relatórios do sistema. Balancete até então ok, mas necessário ajustar o leiaute, e corrigir o balanço. Verificar total da conta sintética, adicionar valor de "saldo inicial do ano". Relatório de balanço por ano atual e ano anterior.</t>
-  </si>
-  <si>
     <t>Custo em planilha</t>
   </si>
   <si>
@@ -240,6 +237,9 @@
   </si>
   <si>
     <t>Criar e emitir relatórios dos custos</t>
+  </si>
+  <si>
+    <t>Verificar total da conta sintética, assunto tratado em chamado em aberto. Relatório de balanço por ano atual e ano anterior, que a princípio não funcionou, por depender da declaração explícita do ano no relatório. Adicionar valor de "saldo inicial do ano", para isso necessário criar métrica que o contemple.</t>
   </si>
 </sst>
 </file>
@@ -836,7 +836,7 @@
         <v>12</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="G3" s="1"/>
       <c r="AB3" s="5" t="s">
@@ -955,10 +955,10 @@
         <v>2</v>
       </c>
       <c r="B8" s="25" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D8" s="23" t="s">
         <v>44</v>
@@ -967,7 +967,7 @@
         <v>12</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G8" s="1"/>
       <c r="AC8" s="6"/>
@@ -993,7 +993,7 @@
       </c>
       <c r="G9" s="1"/>
     </row>
-    <row r="10" spans="1:29" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:29" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="22" t="s">
         <v>2</v>
       </c>
@@ -1014,7 +1014,7 @@
       </c>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>3</v>
       </c>
@@ -1035,7 +1035,7 @@
       </c>
       <c r="G11" s="1"/>
     </row>
-    <row r="12" spans="1:29" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:29" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
         <v>3</v>
       </c>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="G12" s="1"/>
     </row>
-    <row r="13" spans="1:29" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
att DRE, balanço e refatoração de modelo e ETL pneus
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -116,9 +116,6 @@
     <t>Criar relatórios e indicadores para análise dos custos da operação de transporte.</t>
   </si>
   <si>
-    <t>Aguardando fim do projeto de melhoria de pneus.</t>
-  </si>
-  <si>
     <t>CRM</t>
   </si>
   <si>
@@ -221,9 +218,6 @@
     <t>Após solicitação da Raquel para alterar a data de referência, do fim da oportunidade para o início, não há mais pendências.</t>
   </si>
   <si>
-    <t>Painel DRE entregue, e utilizado em reunião de diretoria referente a maio.</t>
-  </si>
-  <si>
     <t>Após nova avaliação, a OS portuária já possui campos de motorista, CM e SR, porém não é claro qual o processo de alimentação dessas informações.</t>
   </si>
   <si>
@@ -239,7 +233,13 @@
     <t>Criar e emitir relatórios dos custos</t>
   </si>
   <si>
-    <t>Verificar total da conta sintética, assunto tratado em chamado em aberto. Relatório de balanço por ano atual e ano anterior, que a princípio não funcionou, por depender da declaração explícita do ano no relatório. Adicionar valor de "saldo inicial do ano", para isso necessário criar métrica que o contemple.</t>
+    <t>Alterados modelo e ETL para carregar novo modelo de dados de pneus. Criar relatórios, avaliá-los e disponibilizá-los para uso junto aos painéis de manutenção e combustível.</t>
+  </si>
+  <si>
+    <t>Painel DRE entregue, e utilizado em reunião de diretoria referente a maio. Realizar manutenção na conta 331803002, que está divergente do valor esperado das despesas operacionais.</t>
+  </si>
+  <si>
+    <t>Adicionar valor de "saldo inicial do ano", pendente de métrica que o contemple. Formatar os número conforme os da DRE e disponibilizar relatórios de balanço.</t>
   </si>
 </sst>
 </file>
@@ -789,10 +789,10 @@
         <v>8</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="2" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:29" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
@@ -803,13 +803,13 @@
         <v>25</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E2" s="14" t="s">
         <v>12</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="G2" s="1"/>
       <c r="AB2" s="5" t="s">
@@ -819,7 +819,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:29" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>1</v>
       </c>
@@ -854,16 +854,16 @@
         <v>18</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E4" s="23" t="s">
         <v>14</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G4" s="1"/>
       <c r="AB4" s="5" t="s">
@@ -881,10 +881,10 @@
         <v>19</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E5" s="23" t="s">
         <v>14</v>
@@ -894,7 +894,7 @@
       </c>
       <c r="G5" s="1"/>
       <c r="AB5" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="AC5" s="5" t="s">
         <v>13</v>
@@ -908,20 +908,20 @@
         <v>20</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E6" s="23" t="s">
         <v>14</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G6" s="1"/>
       <c r="AB6" s="5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="AC6" s="5"/>
     </row>
@@ -933,7 +933,7 @@
         <v>21</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D7" s="23" t="s">
         <v>10</v>
@@ -942,11 +942,11 @@
         <v>14</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G7" s="1"/>
       <c r="AB7" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="AC7" s="5"/>
     </row>
@@ -955,19 +955,19 @@
         <v>2</v>
       </c>
       <c r="B8" s="25" t="s">
+        <v>65</v>
+      </c>
+      <c r="C8" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="24" t="s">
-        <v>69</v>
-      </c>
       <c r="D8" s="23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E8" s="23" t="s">
         <v>12</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G8" s="1"/>
       <c r="AC8" s="6"/>
@@ -977,19 +977,19 @@
         <v>2</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>27</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E9" s="23" t="s">
         <v>13</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G9" s="1"/>
     </row>
@@ -998,40 +998,40 @@
         <v>2</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E10" s="23" t="s">
         <v>13</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:29" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>3</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C11" s="20" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="E11" s="16" t="s">
         <v>14</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="G11" s="1"/>
     </row>
@@ -1040,19 +1040,19 @@
         <v>3</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E12" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G12" s="1"/>
     </row>
@@ -1061,10 +1061,10 @@
         <v>3</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>6</v>
@@ -1073,7 +1073,7 @@
         <v>12</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G13" s="1"/>
       <c r="J13" s="26"/>
@@ -1084,10 +1084,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D14" s="16" t="s">
         <v>9</v>
@@ -1096,18 +1096,18 @@
         <v>12</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="19" t="s">
         <v>46</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>47</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>9</v>
@@ -1116,18 +1116,18 @@
         <v>13</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:29" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B16" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" s="19" t="s">
         <v>59</v>
-      </c>
-      <c r="C16" s="19" t="s">
-        <v>60</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>9</v>
@@ -1136,7 +1136,7 @@
         <v>14</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1150,38 +1150,38 @@
         <v>24</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E17" s="17" t="s">
         <v>13</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C18" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="B18" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="C18" s="21" t="s">
-        <v>31</v>
-      </c>
       <c r="D18" s="17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E18" s="17" t="s">
         <v>13</v>
       </c>
       <c r="F18" s="21" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B19" s="12" t="s">
         <v>23</v>
@@ -1190,13 +1190,13 @@
         <v>24</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E19" s="17" t="s">
         <v>14</v>
       </c>
       <c r="F19" s="21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
planilha diária de indicadores e energia do Bardella
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -149,9 +149,6 @@
     <t>Automatizar informações manuais da planilha</t>
   </si>
   <si>
-    <t>A partir da NF recebida mensalmente é possível registrar o abastecimento de energia, com kWh, valor, horímetro e horas rodadas. Criar posto e produto energia elétrica do Bardella, vincular tipo de combustível (energia) ao produto, testar a movimentação e o cálculo da média.</t>
-  </si>
-  <si>
     <t>em pausa</t>
   </si>
   <si>
@@ -194,9 +191,6 @@
     <t>O projeto Fast Analytics não atenderia à necessidade, conforme análise do Paulino. Cristianne também sinalizou manter a planilha, já que sua substituição não seria viável nem pelo RM, após análise das duas soluções.</t>
   </si>
   <si>
-    <t>Conforme solicitado pelo Wellington em reunião quinzenal, criar um método de carga automática dos dados de disponibilidade, veículos aguardando peças e em serviços externos, que hoje são informações manualmente preenchidas para a reunião mensal. Projeto de criação de planilha preenchida pelo setor de manutenção com um leiaute específico para a carga junto das demais informações do setor, como OS realizadas e abastecimentos.</t>
-  </si>
-  <si>
     <t>indicadores</t>
   </si>
   <si>
@@ -240,6 +234,12 @@
   </si>
   <si>
     <t>Adicionar valor de "saldo inicial do ano", pendente de métrica que o contemple. Formatar os número conforme os da DRE e disponibilizar relatórios de balanço.</t>
+  </si>
+  <si>
+    <t>A partir da NF recebida mensalmente é possível registrar o abastecimento de energia, com kWh, valor, horímetro e horas rodadas. Criar posto e produto energia elétrica do Bardella, vincular tipo de combustível (energia) ao produto, testar a movimentação e o cálculo da média. Aguardando definição do início do processo pelo Wellington.</t>
+  </si>
+  <si>
+    <t>Conforme solicitado pelo Wellington em reunião quinzenal, criar um padrão dos dados de disponibilidade, veículos aguardando peças e em serviços externos, que hoje são informações manualmente preenchidas para a reunião mensal. Planilha modelo criada e colocada no drive, para disponibilizar à manutenção para preenchimento diário. Analisar um método para automatizar a carga da planilha.</t>
   </si>
 </sst>
 </file>
@@ -803,13 +803,13 @@
         <v>25</v>
       </c>
       <c r="D2" s="14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E2" s="14" t="s">
         <v>12</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G2" s="1"/>
       <c r="AB2" s="5" t="s">
@@ -836,7 +836,7 @@
         <v>12</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G3" s="1"/>
       <c r="AB3" s="5" t="s">
@@ -857,13 +857,13 @@
         <v>31</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E4" s="23" t="s">
         <v>14</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G4" s="1"/>
       <c r="AB4" s="5" t="s">
@@ -884,7 +884,7 @@
         <v>38</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E5" s="23" t="s">
         <v>14</v>
@@ -894,7 +894,7 @@
       </c>
       <c r="G5" s="1"/>
       <c r="AB5" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AC5" s="5" t="s">
         <v>13</v>
@@ -911,17 +911,17 @@
         <v>38</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E6" s="23" t="s">
         <v>14</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G6" s="1"/>
       <c r="AB6" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="AC6" s="5"/>
     </row>
@@ -942,11 +942,11 @@
         <v>14</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G7" s="1"/>
       <c r="AB7" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="AC7" s="5"/>
     </row>
@@ -955,19 +955,19 @@
         <v>2</v>
       </c>
       <c r="B8" s="25" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="24" t="s">
         <v>65</v>
       </c>
-      <c r="C8" s="24" t="s">
-        <v>67</v>
-      </c>
       <c r="D8" s="23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E8" s="23" t="s">
         <v>12</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G8" s="1"/>
       <c r="AC8" s="6"/>
@@ -977,19 +977,19 @@
         <v>2</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>27</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E9" s="23" t="s">
         <v>13</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G9" s="1"/>
     </row>
@@ -1004,13 +1004,13 @@
         <v>39</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E10" s="23" t="s">
         <v>13</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G10" s="1"/>
     </row>
@@ -1019,7 +1019,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C11" s="20" t="s">
         <v>16</v>
@@ -1031,7 +1031,7 @@
         <v>14</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="G11" s="1"/>
     </row>
@@ -1046,17 +1046,17 @@
         <v>33</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E12" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G12" s="1"/>
     </row>
-    <row r="13" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
         <v>3</v>
       </c>
@@ -1064,7 +1064,7 @@
         <v>35</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>6</v>
@@ -1073,7 +1073,7 @@
         <v>12</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="G13" s="1"/>
       <c r="J13" s="26"/>
@@ -1096,18 +1096,18 @@
         <v>12</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>40</v>
+        <v>69</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="19" t="s">
         <v>45</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>46</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>9</v>
@@ -1116,18 +1116,18 @@
         <v>13</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="16" spans="1:29" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="16" spans="1:29" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>9</v>
@@ -1136,7 +1136,7 @@
         <v>14</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1150,13 +1150,13 @@
         <v>24</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E17" s="17" t="s">
         <v>13</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1170,18 +1170,18 @@
         <v>30</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E18" s="17" t="s">
         <v>13</v>
       </c>
       <c r="F18" s="21" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B19" s="12" t="s">
         <v>23</v>
@@ -1190,13 +1190,13 @@
         <v>24</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E19" s="17" t="s">
         <v>14</v>
       </c>
       <c r="F19" s="21" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
att custo TMS e compras
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -113,9 +113,6 @@
     <t>Adequar indicadores do projeto TMS</t>
   </si>
   <si>
-    <t>Criar relatórios e indicadores para análise dos custos da operação de transporte.</t>
-  </si>
-  <si>
     <t>CRM</t>
   </si>
   <si>
@@ -167,15 +164,6 @@
     <t>Levantar a relação de motoristas e contêineres vazios devolvidos</t>
   </si>
   <si>
-    <t>Criar relatórios e indicadores para análise dos custos dos veículos da operação de transporte. Pendente validação das informações já existentes do custo dos veículos, antes de sua apropriação à viagens.</t>
-  </si>
-  <si>
-    <t>Criar relatórios e indicadores para análise do custo com pessoal da operação de transporte.</t>
-  </si>
-  <si>
-    <t>Adequar relatórios referentes à performance de atendimento, à movimentação de carga e a outras informações relevantes para a operação de transporte.</t>
-  </si>
-  <si>
     <t>Compras</t>
   </si>
   <si>
@@ -185,9 +173,6 @@
     <t>Automatizar carga de dados não controlados pelo sistema</t>
   </si>
   <si>
-    <t>Criar relatórios e indicadores da receita da operação de transporte. Necessário modelar a obtenção das receitas extras das viagens, como aquelas de RPS e nota de débito, e criar relatórios que confirmem essas informações ou não.</t>
-  </si>
-  <si>
     <t>O projeto Fast Analytics não atenderia à necessidade, conforme análise do Paulino. Cristianne também sinalizou manter a planilha, já que sua substituição não seria viável nem pelo RM, após análise das duas soluções.</t>
   </si>
   <si>
@@ -206,9 +191,6 @@
     <t>Os custos são apropriados de acordo com rotina customizada no módulo de faturamento. A validação e a análise dos valores, pela contabilidade, apoia-se em relatórios existentes ou criados com essa finalidade, e são disponibilizados nos cubos do RM.</t>
   </si>
   <si>
-    <t>Conforme demanda do Manoel Junior, os relatórios são criados ou emitidos junto com a Fátima.</t>
-  </si>
-  <si>
     <t>Após solicitação da Raquel para alterar a data de referência, do fim da oportunidade para o início, não há mais pendências.</t>
   </si>
   <si>
@@ -221,9 +203,6 @@
     <t>Custo em planilha</t>
   </si>
   <si>
-    <t>Conforme demanda do analista de custos (Paulo Cesar) por relatórios por ele compilados para criar o custo do TMS em Excel.</t>
-  </si>
-  <si>
     <t>Criar e emitir relatórios dos custos</t>
   </si>
   <si>
@@ -240,6 +219,27 @@
   </si>
   <si>
     <t>Balanço e balancete entregues.</t>
+  </si>
+  <si>
+    <t>Criar relatórios e indicadores da receita da operação de transporte. Necessário modelar a obtenção das receitas extras das viagens, como aquelas de RPS e nota de débito, e criar relatórios que confirmem essas informações ou não. Pausa solicitada pelo Porto.</t>
+  </si>
+  <si>
+    <t>Criar relatórios e indicadores para análise dos custos da operação de transporte. Pausa solicitada pelo Porto.</t>
+  </si>
+  <si>
+    <t>Criar relatórios e indicadores para análise dos custos dos veículos da operação de transporte. Pendente validação das informações já existentes do custo dos veículos, antes de sua apropriação à viagens. Pausa solicitada pelo Porto.</t>
+  </si>
+  <si>
+    <t>Criar relatórios e indicadores para análise do custo com pessoal da operação de transporte. Pausa solicitada pelo Porto.</t>
+  </si>
+  <si>
+    <t>Adequar relatórios referentes à performance de atendimento, à movimentação de carga e a outras informações relevantes para a operação de transporte. Pausa solicitada pelo Porto.</t>
+  </si>
+  <si>
+    <t>Conforme demanda do analista de custos (Paulo Cesar) por emissão relatórios para que ele compile o custo do TMS em Excel.</t>
+  </si>
+  <si>
+    <t>Conforme demanda do Manoel Junior, os relatórios são criados ou emitidos junto com a Fátima. Filtrados os fornecedores não pertinentes à análise de suprimentos (RDB, VR etc.), pendente análise da Fátima e do Manoel Jr.</t>
   </si>
 </sst>
 </file>
@@ -789,7 +789,7 @@
         <v>8</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:29" ht="30" x14ac:dyDescent="0.25">
@@ -809,7 +809,7 @@
         <v>12</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="G2" s="1"/>
       <c r="AB2" s="5" t="s">
@@ -830,13 +830,13 @@
         <v>26</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E3" s="14" t="s">
         <v>12</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="G3" s="1"/>
       <c r="AB3" s="5" t="s">
@@ -854,16 +854,16 @@
         <v>18</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E4" s="23" t="s">
         <v>14</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="G4" s="1"/>
       <c r="AB4" s="5" t="s">
@@ -881,20 +881,20 @@
         <v>19</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E5" s="23" t="s">
         <v>14</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>28</v>
+        <v>65</v>
       </c>
       <c r="G5" s="1"/>
       <c r="AB5" s="5" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="AC5" s="5" t="s">
         <v>13</v>
@@ -908,20 +908,20 @@
         <v>20</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E6" s="23" t="s">
         <v>14</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="G6" s="1"/>
       <c r="AB6" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="AC6" s="5"/>
     </row>
@@ -933,7 +933,7 @@
         <v>21</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D7" s="23" t="s">
         <v>10</v>
@@ -942,11 +942,11 @@
         <v>14</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>47</v>
+        <v>67</v>
       </c>
       <c r="G7" s="1"/>
       <c r="AB7" s="6" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AC7" s="5"/>
     </row>
@@ -955,19 +955,19 @@
         <v>2</v>
       </c>
       <c r="B8" s="25" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E8" s="23" t="s">
         <v>12</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="G8" s="1"/>
       <c r="AC8" s="6"/>
@@ -977,19 +977,19 @@
         <v>2</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>27</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E9" s="23" t="s">
         <v>13</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="G9" s="1"/>
     </row>
@@ -998,19 +998,19 @@
         <v>2</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E10" s="23" t="s">
         <v>13</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="G10" s="1"/>
     </row>
@@ -1019,7 +1019,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C11" s="20" t="s">
         <v>16</v>
@@ -1031,7 +1031,7 @@
         <v>14</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="G11" s="1"/>
     </row>
@@ -1040,19 +1040,19 @@
         <v>3</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E12" s="16" t="s">
         <v>12</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="G12" s="1"/>
     </row>
@@ -1061,10 +1061,10 @@
         <v>3</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>6</v>
@@ -1073,7 +1073,7 @@
         <v>12</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="G13" s="1"/>
       <c r="J13" s="26"/>
@@ -1084,10 +1084,10 @@
         <v>3</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D14" s="16" t="s">
         <v>9</v>
@@ -1096,18 +1096,18 @@
         <v>12</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="19" t="s">
         <v>44</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>45</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>9</v>
@@ -1116,18 +1116,18 @@
         <v>13</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" spans="1:29" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C16" s="19" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>9</v>
@@ -1136,7 +1136,7 @@
         <v>14</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1150,38 +1150,38 @@
         <v>24</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E17" s="17" t="s">
         <v>13</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
+        <v>28</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="C18" s="21" t="s">
-        <v>30</v>
-      </c>
       <c r="D18" s="17" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E18" s="17" t="s">
         <v>13</v>
       </c>
       <c r="F18" s="21" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B19" s="12" t="s">
         <v>23</v>
@@ -1190,13 +1190,13 @@
         <v>24</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>42</v>
+        <v>9</v>
       </c>
       <c r="E19" s="17" t="s">
         <v>14</v>
       </c>
       <c r="F19" s="21" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
att compras e custo TMS
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -221,6 +221,9 @@
     <t>Balanço e balancete entregues.</t>
   </si>
   <si>
+    <t>Conforme demanda do Manoel Junior, os relatórios são criados ou emitidos junto com a Fátima. Filtrados os fornecedores não pertinentes à análise de suprimentos (RDB, VR etc.)</t>
+  </si>
+  <si>
     <t>Criar relatórios e indicadores da receita da operação de transporte. Necessário modelar a obtenção das receitas extras das viagens, como aquelas de RPS e nota de débito, e criar relatórios que confirmem essas informações ou não. Pausa solicitada pelo Porto.</t>
   </si>
   <si>
@@ -233,13 +236,10 @@
     <t>Criar relatórios e indicadores para análise do custo com pessoal da operação de transporte. Pausa solicitada pelo Porto.</t>
   </si>
   <si>
+    <t>Conforme demanda do analista de custos (Paulo Cesar) por relatórios por ele compilados para criar o custo do TMS em Excel. Pausa solicitada pelo Porto.</t>
+  </si>
+  <si>
     <t>Adequar relatórios referentes à performance de atendimento, à movimentação de carga e a outras informações relevantes para a operação de transporte. Pausa solicitada pelo Porto.</t>
-  </si>
-  <si>
-    <t>Conforme demanda do analista de custos (Paulo Cesar) por emissão relatórios para que ele compile o custo do TMS em Excel.</t>
-  </si>
-  <si>
-    <t>Conforme demanda do Manoel Junior, os relatórios são criados ou emitidos junto com a Fátima. Filtrados os fornecedores não pertinentes à análise de suprimentos (RDB, VR etc.), pendente análise da Fátima e do Manoel Jr.</t>
   </si>
 </sst>
 </file>
@@ -863,7 +863,7 @@
         <v>14</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="G4" s="1"/>
       <c r="AB4" s="5" t="s">
@@ -890,7 +890,7 @@
         <v>14</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G5" s="1"/>
       <c r="AB5" s="5" t="s">
@@ -917,7 +917,7 @@
         <v>14</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G6" s="1"/>
       <c r="AB6" s="5" t="s">
@@ -942,7 +942,7 @@
         <v>14</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G7" s="1"/>
       <c r="AB7" s="6" t="s">
@@ -989,7 +989,7 @@
         <v>13</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="G9" s="1"/>
     </row>
@@ -1196,7 +1196,7 @@
         <v>14</v>
       </c>
       <c r="F19" s="21" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
com o fim do projeto de pneus, criar os indicadores
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="70">
   <si>
     <t>projeto</t>
   </si>
@@ -57,9 +57,6 @@
   </si>
   <si>
     <t>aguardando usuário</t>
-  </si>
-  <si>
-    <t>a iniciar</t>
   </si>
   <si>
     <t>prioridade</t>
@@ -777,19 +774,19 @@
         <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:29" ht="30" x14ac:dyDescent="0.25">
@@ -800,23 +797,23 @@
         <v>7</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>6</v>
       </c>
       <c r="E2" s="14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G2" s="1"/>
       <c r="AB2" s="5" t="s">
         <v>5</v>
       </c>
       <c r="AC2" s="5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
@@ -824,26 +821,26 @@
         <v>1</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D3" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E3" s="14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G3" s="1"/>
       <c r="AB3" s="5" t="s">
         <v>9</v>
       </c>
       <c r="AC3" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -851,26 +848,26 @@
         <v>2</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C4" s="24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E4" s="23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G4" s="1"/>
       <c r="AB4" s="5" t="s">
         <v>6</v>
       </c>
       <c r="AC4" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:29" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -878,26 +875,26 @@
         <v>2</v>
       </c>
       <c r="B5" s="25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C5" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G5" s="1"/>
       <c r="AB5" s="5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AC5" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:29" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -905,23 +902,23 @@
         <v>2</v>
       </c>
       <c r="B6" s="25" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E6" s="23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G6" s="1"/>
       <c r="AB6" s="5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="AC6" s="5"/>
     </row>
@@ -930,23 +927,23 @@
         <v>2</v>
       </c>
       <c r="B7" s="25" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C7" s="24" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="E7" s="23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G7" s="1"/>
       <c r="AB7" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="AC7" s="5"/>
     </row>
@@ -955,19 +952,19 @@
         <v>2</v>
       </c>
       <c r="B8" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="24" t="s">
-        <v>58</v>
-      </c>
       <c r="D8" s="23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E8" s="23" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="G8" s="1"/>
       <c r="AC8" s="6"/>
@@ -977,19 +974,19 @@
         <v>2</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E9" s="23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G9" s="1"/>
     </row>
@@ -998,19 +995,19 @@
         <v>2</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E10" s="23" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G10" s="1"/>
     </row>
@@ -1019,19 +1016,19 @@
         <v>3</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D11" s="16" t="s">
         <v>6</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G11" s="1"/>
     </row>
@@ -1040,19 +1037,19 @@
         <v>3</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G12" s="1"/>
     </row>
@@ -1061,19 +1058,19 @@
         <v>3</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>6</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G13" s="1"/>
       <c r="J13" s="26"/>
@@ -1084,119 +1081,119 @@
         <v>3</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C14" s="20" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B15" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="C15" s="19" t="s">
         <v>43</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>44</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>9</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:29" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B16" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C16" s="19" t="s">
         <v>51</v>
-      </c>
-      <c r="C16" s="19" t="s">
-        <v>52</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>9</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B17" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B17" s="12" t="s">
+      <c r="C17" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="C17" s="21" t="s">
-        <v>24</v>
-      </c>
       <c r="D17" s="17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C18" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="B18" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="21" t="s">
-        <v>29</v>
-      </c>
       <c r="D18" s="17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F18" s="21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B19" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C19" s="21" t="s">
         <v>23</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>24</v>
       </c>
       <c r="D19" s="17" t="s">
         <v>9</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F19" s="21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
alteração da consulta análise para CPK pneus
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -203,15 +203,9 @@
     <t>Criar e emitir relatórios dos custos</t>
   </si>
   <si>
-    <t>Alterados modelo e ETL para carregar novo modelo de dados de pneus. Criar relatórios, avaliá-los e disponibilizá-los para uso junto aos painéis de manutenção e combustível.</t>
-  </si>
-  <si>
     <t>A partir da NF recebida mensalmente é possível registrar o abastecimento de energia, com kWh, valor, horímetro e horas rodadas. Criar posto e produto energia elétrica do Bardella, vincular tipo de combustível (energia) ao produto, testar a movimentação e o cálculo da média. Aguardando definição do início do processo pelo Wellington.</t>
   </si>
   <si>
-    <t>Conforme solicitado pelo Wellington em reunião quinzenal, criar um padrão dos dados de disponibilidade, veículos aguardando peças e em serviços externos, que hoje são informações manualmente preenchidas para a reunião mensal. Planilha modelo criada e colocada no drive, para disponibilizar à manutenção para preenchimento diário. Analisar um método para automatizar a carga da planilha.</t>
-  </si>
-  <si>
     <t>Painel DRE entregue, e utilizado em reunião de diretoria referente a maio. Tratar a característica ambígua credora e devedora da conta 331803, para que exiba valor positivo ou negativo quando pertinente.</t>
   </si>
   <si>
@@ -233,10 +227,16 @@
     <t>Criar relatórios e indicadores para análise do custo com pessoal da operação de transporte. Pausa solicitada pelo Porto.</t>
   </si>
   <si>
-    <t>Conforme demanda do analista de custos (Paulo Cesar) por relatórios por ele compilados para criar o custo do TMS em Excel. Pausa solicitada pelo Porto.</t>
-  </si>
-  <si>
     <t>Adequar relatórios referentes à performance de atendimento, à movimentação de carga e a outras informações relevantes para a operação de transporte. Pausa solicitada pelo Porto.</t>
+  </si>
+  <si>
+    <t>Conforme demanda do analista de custos (Paulo Cesar) por relatórios por ele compilados para criar o custo do TMS em Excel.</t>
+  </si>
+  <si>
+    <t>Alterados modelo e ETL para carregar novo modelo de dados de pneus. Criar relatórios, avaliá-los e disponibilizá-los para uso junto aos painéis de manutenção e combustível. Iminente disponibilização de painel de exemplo.</t>
+  </si>
+  <si>
+    <t>Conforme solicitado pelo Wellington em reunião quinzenal, criar um padrão dos dados de disponibilidade, veículos aguardando peças e em serviços externos, que hoje são informações manualmente preenchidas para a reunião mensal. Planilha modelo criada, disponibilizada no drive para as equipes de manutenção e aperfeiçoada pelo Stefson para viabilizar a carga automática dos dados.</t>
   </si>
 </sst>
 </file>
@@ -806,7 +806,7 @@
         <v>11</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="G2" s="1"/>
       <c r="AB2" s="5" t="s">
@@ -833,7 +833,7 @@
         <v>11</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="G3" s="1"/>
       <c r="AB3" s="5" t="s">
@@ -860,7 +860,7 @@
         <v>13</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="G4" s="1"/>
       <c r="AB4" s="5" t="s">
@@ -887,7 +887,7 @@
         <v>13</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="G5" s="1"/>
       <c r="AB5" s="5" t="s">
@@ -914,7 +914,7 @@
         <v>13</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="G6" s="1"/>
       <c r="AB6" s="5" t="s">
@@ -939,7 +939,7 @@
         <v>13</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="G7" s="1"/>
       <c r="AB7" s="6" t="s">
@@ -964,7 +964,7 @@
         <v>11</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G8" s="1"/>
       <c r="AC8" s="6"/>
@@ -986,7 +986,7 @@
         <v>12</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="G9" s="1"/>
     </row>
@@ -1028,7 +1028,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G11" s="1"/>
     </row>
@@ -1070,7 +1070,7 @@
         <v>11</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="G13" s="1"/>
       <c r="J13" s="26"/>
@@ -1093,7 +1093,7 @@
         <v>11</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1193,7 +1193,7 @@
         <v>13</v>
       </c>
       <c r="F19" s="21" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
projetos: op portuária, pneus
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -185,9 +185,6 @@
     <t>Otimizar a análise do custo da operação portuária</t>
   </si>
   <si>
-    <t>Os custos são apropriados de acordo com rotina customizada no módulo de faturamento. A validação e a análise dos valores, pela contabilidade, apoia-se em relatórios existentes ou criados com essa finalidade, e são disponibilizados nos cubos do RM.</t>
-  </si>
-  <si>
     <t>Após solicitação da Raquel para alterar a data de referência, do fim da oportunidade para o início, não há mais pendências.</t>
   </si>
   <si>
@@ -233,10 +230,13 @@
     <t>Conforme demanda do analista de custos (Paulo Cesar) por relatórios por ele compilados para criar o custo do TMS em Excel.</t>
   </si>
   <si>
-    <t>Alterados modelo e ETL para carregar novo modelo de dados de pneus. Criar relatórios, avaliá-los e disponibilizá-los para uso junto aos painéis de manutenção e combustível. Iminente disponibilização de painel de exemplo.</t>
-  </si>
-  <si>
     <t>Conforme solicitado pelo Wellington em reunião quinzenal, criar um padrão dos dados de disponibilidade, veículos aguardando peças e em serviços externos, que hoje são informações manualmente preenchidas para a reunião mensal. Planilha modelo criada, disponibilizada no drive para as equipes de manutenção e aperfeiçoada pelo Stefson para viabilizar a carga automática dos dados.</t>
+  </si>
+  <si>
+    <t>Em reunião com Silvio, os relatórios foram aprovados, e o desenvolvimento fica sob demanda.</t>
+  </si>
+  <si>
+    <t>Conforme demanda da análise do custo, pelo Paulo Cesar, Porto, Cristianne. Aprovado projeto de melhoria das rotinas customizadas do custo da operação portuária.</t>
   </si>
 </sst>
 </file>
@@ -806,7 +806,7 @@
         <v>11</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G2" s="1"/>
       <c r="AB2" s="5" t="s">
@@ -833,7 +833,7 @@
         <v>11</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G3" s="1"/>
       <c r="AB3" s="5" t="s">
@@ -860,7 +860,7 @@
         <v>13</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G4" s="1"/>
       <c r="AB4" s="5" t="s">
@@ -887,7 +887,7 @@
         <v>13</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G5" s="1"/>
       <c r="AB5" s="5" t="s">
@@ -914,7 +914,7 @@
         <v>13</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G6" s="1"/>
       <c r="AB6" s="5" t="s">
@@ -939,7 +939,7 @@
         <v>13</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G7" s="1"/>
       <c r="AB7" s="6" t="s">
@@ -952,10 +952,10 @@
         <v>2</v>
       </c>
       <c r="B8" s="25" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="24" t="s">
         <v>56</v>
-      </c>
-      <c r="C8" s="24" t="s">
-        <v>57</v>
       </c>
       <c r="D8" s="23" t="s">
         <v>40</v>
@@ -964,7 +964,7 @@
         <v>11</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G8" s="1"/>
       <c r="AC8" s="6"/>
@@ -986,7 +986,7 @@
         <v>12</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G9" s="1"/>
     </row>
@@ -1011,7 +1011,7 @@
       </c>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
         <v>3</v>
       </c>
@@ -1022,7 +1022,7 @@
         <v>15</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>6</v>
+        <v>40</v>
       </c>
       <c r="E11" s="16" t="s">
         <v>11</v>
@@ -1049,7 +1049,7 @@
         <v>11</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G12" s="1"/>
     </row>
@@ -1070,7 +1070,7 @@
         <v>11</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G13" s="1"/>
       <c r="J13" s="26"/>
@@ -1093,7 +1093,7 @@
         <v>11</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1113,7 +1113,7 @@
         <v>12</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="16" spans="1:29" ht="30" x14ac:dyDescent="0.25">
@@ -1127,13 +1127,13 @@
         <v>51</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="E16" s="15" t="s">
         <v>13</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>52</v>
+        <v>69</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1173,7 +1173,7 @@
         <v>12</v>
       </c>
       <c r="F18" s="21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -1187,13 +1187,13 @@
         <v>23</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>9</v>
+        <v>40</v>
       </c>
       <c r="E19" s="17" t="s">
         <v>13</v>
       </c>
       <c r="F19" s="21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
att RH, CRM e compras
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -164,9 +164,6 @@
     <t>Compras</t>
   </si>
   <si>
-    <t>Conforme demanda do setor pessoal.</t>
-  </si>
-  <si>
     <t>Automatizar carga de dados não controlados pelo sistema</t>
   </si>
   <si>
@@ -185,9 +182,6 @@
     <t>Otimizar a análise do custo da operação portuária</t>
   </si>
   <si>
-    <t>Após solicitação da Raquel para alterar a data de referência, do fim da oportunidade para o início, não há mais pendências.</t>
-  </si>
-  <si>
     <t>Após nova avaliação, a OS portuária já possui campos de motorista, CM e SR, porém não é claro qual o processo de alimentação dessas informações.</t>
   </si>
   <si>
@@ -209,9 +203,6 @@
     <t>Balanço e balancete entregues.</t>
   </si>
   <si>
-    <t>Conforme demanda do Manoel Junior, os relatórios são criados ou emitidos junto com a Fátima. Filtrados os fornecedores não pertinentes à análise de suprimentos (RDB, VR etc.)</t>
-  </si>
-  <si>
     <t>Criar relatórios e indicadores da receita da operação de transporte. Necessário modelar a obtenção das receitas extras das viagens, como aquelas de RPS e nota de débito, e criar relatórios que confirmem essas informações ou não. Pausa solicitada pelo Porto.</t>
   </si>
   <si>
@@ -237,6 +228,15 @@
   </si>
   <si>
     <t>Conforme demanda da análise do custo, pelo Paulo Cesar, Porto, Cristianne. Aprovado projeto de melhoria das rotinas customizadas do custo da operação portuária.</t>
+  </si>
+  <si>
+    <t>Conforme demanda do Manoel Junior, os relatórios são criados ou emitidos junto com a Fátima. Filtrados os fornecedores não pertinentes à análise de suprimentos (RDB, VR etc.). Adicionadas informações de solicitações de compras, a fim de possibilitar a análise dessa fase do processo de compras além do pedido de compra.</t>
+  </si>
+  <si>
+    <t>Após solicitação da Raquel para alterar a data de referência, do fim da oportunidade para o início, não há mais pendências. Fausto solicitou adição do valor do produto da oportunidade, e pendente melhoria no módulo para melhor identificar a oportunidades.</t>
+  </si>
+  <si>
+    <t>Conforme demanda do setor pessoal. Planilha de migração do plano Hapvida para Unimed.</t>
   </si>
 </sst>
 </file>
@@ -806,7 +806,7 @@
         <v>11</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="G2" s="1"/>
       <c r="AB2" s="5" t="s">
@@ -833,7 +833,7 @@
         <v>11</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G3" s="1"/>
       <c r="AB3" s="5" t="s">
@@ -860,7 +860,7 @@
         <v>13</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="G4" s="1"/>
       <c r="AB4" s="5" t="s">
@@ -887,7 +887,7 @@
         <v>13</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="G5" s="1"/>
       <c r="AB5" s="5" t="s">
@@ -914,7 +914,7 @@
         <v>13</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="G6" s="1"/>
       <c r="AB6" s="5" t="s">
@@ -939,7 +939,7 @@
         <v>13</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G7" s="1"/>
       <c r="AB7" s="6" t="s">
@@ -952,10 +952,10 @@
         <v>2</v>
       </c>
       <c r="B8" s="25" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D8" s="23" t="s">
         <v>40</v>
@@ -964,7 +964,7 @@
         <v>11</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G8" s="1"/>
       <c r="AC8" s="6"/>
@@ -974,7 +974,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C9" s="24" t="s">
         <v>26</v>
@@ -986,7 +986,7 @@
         <v>12</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G9" s="1"/>
     </row>
@@ -1007,7 +1007,7 @@
         <v>12</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G10" s="1"/>
     </row>
@@ -1016,7 +1016,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C11" s="20" t="s">
         <v>15</v>
@@ -1028,7 +1028,7 @@
         <v>11</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="G11" s="1"/>
     </row>
@@ -1049,7 +1049,7 @@
         <v>11</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="G12" s="1"/>
     </row>
@@ -1061,7 +1061,7 @@
         <v>33</v>
       </c>
       <c r="C13" s="20" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D13" s="16" t="s">
         <v>6</v>
@@ -1070,7 +1070,7 @@
         <v>11</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="G13" s="1"/>
       <c r="J13" s="26"/>
@@ -1093,7 +1093,7 @@
         <v>11</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1113,7 +1113,7 @@
         <v>12</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:29" ht="30" x14ac:dyDescent="0.25">
@@ -1121,10 +1121,10 @@
         <v>41</v>
       </c>
       <c r="B16" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="19" t="s">
         <v>50</v>
-      </c>
-      <c r="C16" s="19" t="s">
-        <v>51</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>40</v>
@@ -1133,7 +1133,7 @@
         <v>13</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1153,10 +1153,10 @@
         <v>12</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="11" t="s">
         <v>27</v>
       </c>
@@ -1173,10 +1173,10 @@
         <v>12</v>
       </c>
       <c r="F18" s="21" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
         <v>44</v>
       </c>
@@ -1193,7 +1193,7 @@
         <v>13</v>
       </c>
       <c r="F19" s="21" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
att operação portuária; anotar itens para agendas 27 e 28
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -182,9 +182,6 @@
     <t>Otimizar a análise do custo da operação portuária</t>
   </si>
   <si>
-    <t>Após nova avaliação, a OS portuária já possui campos de motorista, CM e SR, porém não é claro qual o processo de alimentação dessas informações.</t>
-  </si>
-  <si>
     <t>Incluir gráfico de MDO e de terceiros no painel Frota &gt; Manutenção. Alterar gráfico acumulado da aba "anual".</t>
   </si>
   <si>
@@ -227,9 +224,6 @@
     <t>Em reunião com Silvio, os relatórios foram aprovados, e o desenvolvimento fica sob demanda.</t>
   </si>
   <si>
-    <t>Conforme demanda da análise do custo, pelo Paulo Cesar, Porto, Cristianne. Aprovado projeto de melhoria das rotinas customizadas do custo da operação portuária.</t>
-  </si>
-  <si>
     <t>Conforme demanda do Manoel Junior, os relatórios são criados ou emitidos junto com a Fátima. Filtrados os fornecedores não pertinentes à análise de suprimentos (RDB, VR etc.). Adicionadas informações de solicitações de compras, a fim de possibilitar a análise dessa fase do processo de compras além do pedido de compra.</t>
   </si>
   <si>
@@ -237,6 +231,12 @@
   </si>
   <si>
     <t>Conforme demanda do setor pessoal. Planilha de migração do plano Hapvida para Unimed.</t>
+  </si>
+  <si>
+    <t>Iniciado o projeto da operação portuária dia 6/12. Busca por otimização geral do processo, que deve atender às regras de negócio vigentes na operação, e de acordo com a análise de custos. Verificar com o operacional a viabilidade de abrir uma OS por tipo de serviço.</t>
+  </si>
+  <si>
+    <t>Após nova avaliação, a OS portuária já possui campos de motorista, CM e SR, porém não é claro qual o processo de alimentação dessas informações. Investigar a rotina de impressão da OS, por ser realizada constantemente e sugerir a inclusão dos dados nos itens das OS e, sendo o caso, automatizar a emissão da EIR no momento de impressão da OS para a saída do contêiner e execução do serviço de devolução de vazio.</t>
   </si>
 </sst>
 </file>
@@ -806,7 +806,7 @@
         <v>11</v>
       </c>
       <c r="F2" s="18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G2" s="1"/>
       <c r="AB2" s="5" t="s">
@@ -833,7 +833,7 @@
         <v>11</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G3" s="1"/>
       <c r="AB3" s="5" t="s">
@@ -860,7 +860,7 @@
         <v>13</v>
       </c>
       <c r="F4" s="24" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G4" s="1"/>
       <c r="AB4" s="5" t="s">
@@ -887,7 +887,7 @@
         <v>13</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G5" s="1"/>
       <c r="AB5" s="5" t="s">
@@ -914,7 +914,7 @@
         <v>13</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G6" s="1"/>
       <c r="AB6" s="5" t="s">
@@ -939,7 +939,7 @@
         <v>13</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G7" s="1"/>
       <c r="AB7" s="6" t="s">
@@ -952,10 +952,10 @@
         <v>2</v>
       </c>
       <c r="B8" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="24" t="s">
         <v>53</v>
-      </c>
-      <c r="C8" s="24" t="s">
-        <v>54</v>
       </c>
       <c r="D8" s="23" t="s">
         <v>40</v>
@@ -964,7 +964,7 @@
         <v>11</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G8" s="1"/>
       <c r="AC8" s="6"/>
@@ -986,7 +986,7 @@
         <v>12</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G9" s="1"/>
     </row>
@@ -1022,13 +1022,13 @@
         <v>15</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="E11" s="16" t="s">
         <v>11</v>
       </c>
       <c r="F11" s="20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G11" s="1"/>
     </row>
@@ -1049,7 +1049,7 @@
         <v>11</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G12" s="1"/>
     </row>
@@ -1070,7 +1070,7 @@
         <v>11</v>
       </c>
       <c r="F13" s="20" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G13" s="1"/>
       <c r="J13" s="26"/>
@@ -1093,10 +1093,10 @@
         <v>11</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="15" spans="1:29" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="15" spans="1:29" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
         <v>41</v>
       </c>
@@ -1113,10 +1113,10 @@
         <v>12</v>
       </c>
       <c r="F15" s="19" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="16" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="16" spans="1:29" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
         <v>41</v>
       </c>
@@ -1127,13 +1127,13 @@
         <v>50</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>40</v>
+        <v>6</v>
       </c>
       <c r="E16" s="15" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F16" s="19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1153,7 +1153,7 @@
         <v>12</v>
       </c>
       <c r="F17" s="21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -1173,7 +1173,7 @@
         <v>12</v>
       </c>
       <c r="F18" s="21" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -1193,7 +1193,7 @@
         <v>13</v>
       </c>
       <c r="F19" s="21" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
eliminação da pendência do Bardella
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -15,7 +15,7 @@
     <sheet name="status" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">status!$A$1:$G$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">status!$A$1:$G$13</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="67">
   <si>
     <t>projeto</t>
   </si>
@@ -125,18 +125,12 @@
     <t>Relatórios, gráficos e indicadores dos sistemas de manutenção</t>
   </si>
   <si>
-    <t>Energia do Bardella</t>
-  </si>
-  <si>
     <t>Painéis</t>
   </si>
   <si>
     <t>Planilha logística</t>
   </si>
   <si>
-    <t>Criar controle de consumo de energia e do contador do Bardella</t>
-  </si>
-  <si>
     <t>Possibilitar a análise dos custos da logística</t>
   </si>
   <si>
@@ -191,12 +185,6 @@
     <t>Criar e emitir relatórios dos custos</t>
   </si>
   <si>
-    <t>A partir da NF recebida mensalmente é possível registrar o abastecimento de energia, com kWh, valor, horímetro e horas rodadas. Criar posto e produto energia elétrica do Bardella, vincular tipo de combustível (energia) ao produto, testar a movimentação e o cálculo da média. Aguardando definição do início do processo pelo Wellington.</t>
-  </si>
-  <si>
-    <t>Painel DRE entregue, e utilizado em reunião de diretoria referente a maio. Tratar a característica ambígua credora e devedora da conta 331803, para que exiba valor positivo ou negativo quando pertinente.</t>
-  </si>
-  <si>
     <t>Balanço e balancete entregues.</t>
   </si>
   <si>
@@ -237,6 +225,9 @@
   </si>
   <si>
     <t>Após nova avaliação, a OS portuária já possui campos de motorista, CM e SR, porém não é claro qual o processo de alimentação dessas informações. Investigar a rotina de impressão da OS, por ser realizada constantemente e sugerir a inclusão dos dados nos itens das OS e, sendo o caso, automatizar a emissão da EIR no momento de impressão da OS para a saída do contêiner e execução do serviço de devolução de vazio.</t>
+  </si>
+  <si>
+    <t>Painel DRE entregue, e utilizado em reunião de diretoria referente a maio 2023. Tratar a característica ambígua credora e devedora da conta 331803, para que exiba valor positivo ou negativo quando pertinente.</t>
   </si>
 </sst>
 </file>
@@ -392,7 +383,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -430,9 +421,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -470,6 +458,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -750,13 +753,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AC19"/>
+  <dimension ref="A1:AC18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
     <col min="2" max="2" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="38.7109375" customWidth="1"/>
-    <col min="4" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" customWidth="1"/>
     <col min="5" max="5" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="119.140625" customWidth="1"/>
     <col min="7" max="7" width="119.140625" hidden="1" customWidth="1"/>
@@ -796,17 +799,17 @@
       <c r="B2" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="E2" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="18" t="s">
-        <v>55</v>
+      <c r="F2" s="17" t="s">
+        <v>66</v>
       </c>
       <c r="G2" s="1"/>
       <c r="AB2" s="5" t="s">
@@ -823,17 +826,17 @@
       <c r="B3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="D3" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" s="14" t="s">
+      <c r="D3" s="26" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="F3" s="18" t="s">
-        <v>56</v>
+      <c r="F3" s="17" t="s">
+        <v>52</v>
       </c>
       <c r="G3" s="1"/>
       <c r="AB3" s="5" t="s">
@@ -844,23 +847,23 @@
       </c>
     </row>
     <row r="4" spans="1:29" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="D4" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="E4" s="23" t="s">
+      <c r="D4" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="E4" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="F4" s="24" t="s">
-        <v>57</v>
+      <c r="F4" s="23" t="s">
+        <v>53</v>
       </c>
       <c r="G4" s="1"/>
       <c r="AB4" s="5" t="s">
@@ -871,143 +874,143 @@
       </c>
     </row>
     <row r="5" spans="1:29" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="C5" s="24" t="s">
+      <c r="C5" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="D5" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="E5" s="23" t="s">
+      <c r="E5" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="24" t="s">
-        <v>58</v>
+      <c r="F5" s="23" t="s">
+        <v>54</v>
       </c>
       <c r="G5" s="1"/>
       <c r="AB5" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="AC5" s="5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:29" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="24" t="s">
+      <c r="C6" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="D6" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="E6" s="23" t="s">
+      <c r="E6" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="24" t="s">
-        <v>59</v>
+      <c r="F6" s="23" t="s">
+        <v>55</v>
       </c>
       <c r="G6" s="1"/>
       <c r="AB6" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="AC6" s="5"/>
     </row>
     <row r="7" spans="1:29" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C7" s="23" t="s">
+        <v>34</v>
+      </c>
+      <c r="D7" s="27" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="E7" s="23" t="s">
+      <c r="E7" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="F7" s="24" t="s">
-        <v>60</v>
+      <c r="F7" s="23" t="s">
+        <v>56</v>
       </c>
       <c r="G7" s="1"/>
       <c r="AB7" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="AC7" s="5"/>
     </row>
     <row r="8" spans="1:29" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="C8" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="D8" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="E8" s="23" t="s">
+      <c r="B8" s="24" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="D8" s="27" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="F8" s="24" t="s">
-        <v>62</v>
+      <c r="F8" s="23" t="s">
+        <v>58</v>
       </c>
       <c r="G8" s="1"/>
       <c r="AC8" s="6"/>
     </row>
     <row r="9" spans="1:29" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="25" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="24" t="s">
+      <c r="B9" s="24" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="27" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="23" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9" s="1"/>
+    </row>
+    <row r="10" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="24" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="E9" s="23" t="s">
+      <c r="E10" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="24" t="s">
-        <v>61</v>
-      </c>
-      <c r="G9" s="1"/>
-    </row>
-    <row r="10" spans="1:29" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="22" t="s">
-        <v>2</v>
-      </c>
-      <c r="B10" s="25" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" s="24" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="E10" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="24" t="s">
-        <v>46</v>
+      <c r="F10" s="23" t="s">
+        <v>44</v>
       </c>
       <c r="G10" s="1"/>
     </row>
@@ -1016,19 +1019,19 @@
         <v>3</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C11" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="F11" s="20" t="s">
-        <v>64</v>
+      <c r="F11" s="19" t="s">
+        <v>60</v>
       </c>
       <c r="G11" s="1"/>
     </row>
@@ -1037,19 +1040,19 @@
         <v>3</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="E12" s="16" t="s">
+      <c r="D12" s="28" t="s">
+        <v>38</v>
+      </c>
+      <c r="E12" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="F12" s="20" t="s">
-        <v>51</v>
+      <c r="F12" s="19" t="s">
+        <v>49</v>
       </c>
       <c r="G12" s="1"/>
     </row>
@@ -1058,154 +1061,134 @@
         <v>3</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C13" s="20" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="E13" s="16" t="s">
+      <c r="E13" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="F13" s="20" t="s">
+      <c r="F13" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="G13" s="1"/>
+      <c r="J13" s="25"/>
+      <c r="L13" s="25"/>
+    </row>
+    <row r="14" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C14" s="18" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="29" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" s="18" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="15" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="29" t="s">
+        <v>6</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="18" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:29" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="D16" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="G13" s="1"/>
-      <c r="J13" s="26"/>
-      <c r="L13" s="26"/>
-    </row>
-    <row r="14" spans="1:29" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B14" s="13" t="s">
+    </row>
+    <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="D14" s="16" t="s">
+      <c r="C17" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" s="30" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="16" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="20" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="15" spans="1:29" ht="60" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B15" s="4" t="s">
+      <c r="E17" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" s="20" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C15" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="D15" s="15" t="s">
-        <v>9</v>
-      </c>
-      <c r="E15" s="15" t="s">
-        <v>12</v>
-      </c>
-      <c r="F15" s="19" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="16" spans="1:29" ht="45" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="C16" s="19" t="s">
-        <v>50</v>
-      </c>
-      <c r="D16" s="15" t="s">
-        <v>6</v>
-      </c>
-      <c r="E16" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="F16" s="19" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" s="12" t="s">
+      <c r="B18" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="C18" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="D17" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="E17" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="F17" s="21" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="C18" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="D18" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="F18" s="21" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A19" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="D19" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="E19" s="17" t="s">
+      <c r="D18" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="E18" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="F19" s="21" t="s">
-        <v>65</v>
+      <c r="F18" s="20" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G14"/>
+  <autoFilter ref="A1:G13"/>
   <sortState ref="AB3:AB8">
     <sortCondition ref="AB3"/>
   </sortState>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E19">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E18">
       <formula1>$AC$3:$AC$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D19">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D18">
       <formula1>$AB$3:$AB$9</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
reorganização para adequar ao projeto da operação portuária
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -15,7 +15,7 @@
     <sheet name="status" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">status!$A$1:$G$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">status!$A$1:$G$9</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="56">
   <si>
     <t>projeto</t>
   </si>
@@ -77,21 +77,9 @@
     <t>Criar indicadores e relatórios de pneus</t>
   </si>
   <si>
-    <t>Balanço</t>
-  </si>
-  <si>
     <t>Receita</t>
   </si>
   <si>
-    <t>Custo viagem</t>
-  </si>
-  <si>
-    <t>Custo veículos</t>
-  </si>
-  <si>
-    <t>Custo pessoal</t>
-  </si>
-  <si>
     <t>RH</t>
   </si>
   <si>
@@ -104,9 +92,6 @@
     <t>Adequar a visão da DRE</t>
   </si>
   <si>
-    <t>Adequar a visão do balanço</t>
-  </si>
-  <si>
     <t>Adequar indicadores do projeto TMS</t>
   </si>
   <si>
@@ -131,18 +116,12 @@
     <t>Planilha logística</t>
   </si>
   <si>
-    <t>Possibilitar a análise dos custos da logística</t>
-  </si>
-  <si>
     <t>Automatizar informações manuais da planilha</t>
   </si>
   <si>
     <t>em pausa</t>
   </si>
   <si>
-    <t>não iniciado</t>
-  </si>
-  <si>
     <t>entregue</t>
   </si>
   <si>
@@ -185,19 +164,7 @@
     <t>Criar e emitir relatórios dos custos</t>
   </si>
   <si>
-    <t>Balanço e balancete entregues.</t>
-  </si>
-  <si>
     <t>Criar relatórios e indicadores da receita da operação de transporte. Necessário modelar a obtenção das receitas extras das viagens, como aquelas de RPS e nota de débito, e criar relatórios que confirmem essas informações ou não. Pausa solicitada pelo Porto.</t>
-  </si>
-  <si>
-    <t>Criar relatórios e indicadores para análise dos custos da operação de transporte. Pausa solicitada pelo Porto.</t>
-  </si>
-  <si>
-    <t>Criar relatórios e indicadores para análise dos custos dos veículos da operação de transporte. Pendente validação das informações já existentes do custo dos veículos, antes de sua apropriação à viagens. Pausa solicitada pelo Porto.</t>
-  </si>
-  <si>
-    <t>Criar relatórios e indicadores para análise do custo com pessoal da operação de transporte. Pausa solicitada pelo Porto.</t>
   </si>
   <si>
     <t>Adequar relatórios referentes à performance de atendimento, à movimentação de carga e a outras informações relevantes para a operação de transporte. Pausa solicitada pelo Porto.</t>
@@ -362,7 +329,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -370,20 +337,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -398,9 +356,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -753,7 +708,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AC18"/>
+  <dimension ref="A1:AC19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
@@ -762,7 +717,7 @@
     <col min="4" max="4" width="10.5703125" customWidth="1"/>
     <col min="5" max="5" width="17.7109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="119.140625" customWidth="1"/>
-    <col min="7" max="7" width="119.140625" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="24.140625" hidden="1" customWidth="1"/>
     <col min="10" max="10" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="9.85546875" bestFit="1" customWidth="1"/>
@@ -789,27 +744,27 @@
         <v>8</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:29" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="17" t="s">
-        <v>24</v>
-      </c>
-      <c r="D2" s="26" t="s">
+      <c r="C2" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="F2" s="17" t="s">
-        <v>66</v>
+      <c r="F2" s="16" t="s">
+        <v>55</v>
       </c>
       <c r="G2" s="1"/>
       <c r="AB2" s="5" t="s">
@@ -819,377 +774,359 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="7" t="s">
+    <row r="3" spans="1:29" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="17" t="s">
-        <v>25</v>
+      <c r="C3" s="22" t="s">
+        <v>24</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>38</v>
-      </c>
-      <c r="E3" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="F3" s="17" t="s">
-        <v>52</v>
+        <v>30</v>
+      </c>
+      <c r="E3" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="22" t="s">
+        <v>45</v>
       </c>
       <c r="G3" s="1"/>
       <c r="AB3" s="5" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="AC3" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="23" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>44</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="E4" s="21" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:29" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="21" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C4" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="D4" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="E4" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="23" t="s">
-        <v>53</v>
+      <c r="F4" s="22" t="s">
+        <v>47</v>
       </c>
       <c r="G4" s="1"/>
       <c r="AB4" s="5" t="s">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="AC4" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:29" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="24" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="D5" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="E5" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="23" t="s">
-        <v>54</v>
+      <c r="B5" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="26" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="22" t="s">
+        <v>46</v>
       </c>
       <c r="G5" s="1"/>
       <c r="AB5" s="5" t="s">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="AC5" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:29" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
+    <row r="6" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="20" t="s">
         <v>2</v>
       </c>
-      <c r="B6" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="E6" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="23" t="s">
-        <v>55</v>
+      <c r="B6" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="26" t="s">
+        <v>31</v>
+      </c>
+      <c r="E6" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="22" t="s">
+        <v>37</v>
       </c>
       <c r="G6" s="1"/>
       <c r="AB6" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="AC6" s="5"/>
-    </row>
-    <row r="7" spans="1:29" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="21" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="23" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="1"/>
+      <c r="AB7" s="5"/>
+    </row>
+    <row r="8" spans="1:29" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="27" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="G8" s="1"/>
+      <c r="AB8" s="5"/>
+    </row>
+    <row r="9" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="27" t="s">
+        <v>6</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" s="1"/>
+      <c r="J9" s="24"/>
+      <c r="L9" s="24"/>
+    </row>
+    <row r="10" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="D7" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" s="22" t="s">
-        <v>13</v>
-      </c>
-      <c r="F7" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="G7" s="1"/>
-      <c r="AB7" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="AC7" s="5"/>
-    </row>
-    <row r="8" spans="1:29" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="21" t="s">
-        <v>2</v>
-      </c>
-      <c r="B8" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="D8" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="E8" s="22" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="23" t="s">
-        <v>58</v>
-      </c>
-      <c r="G8" s="1"/>
-      <c r="AC8" s="6"/>
-    </row>
-    <row r="9" spans="1:29" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="21" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="D9" s="27" t="s">
-        <v>36</v>
-      </c>
-      <c r="E9" s="22" t="s">
+      <c r="D10" s="28" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="G9" s="1"/>
-    </row>
-    <row r="10" spans="1:29" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="21" t="s">
-        <v>2</v>
-      </c>
-      <c r="B10" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="23" t="s">
-        <v>35</v>
-      </c>
-      <c r="D10" s="27" t="s">
-        <v>38</v>
-      </c>
-      <c r="E10" s="22" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="23" t="s">
-        <v>44</v>
-      </c>
-      <c r="G10" s="1"/>
-    </row>
-    <row r="11" spans="1:29" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>15</v>
+      <c r="F10" s="17" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>41</v>
       </c>
       <c r="D11" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="E11" s="15" t="s">
+      <c r="E11" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="F11" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="G11" s="1"/>
-    </row>
-    <row r="12" spans="1:29" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" s="3" t="s">
+      <c r="F11" s="17" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:29" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="19" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" s="28" t="s">
-        <v>38</v>
-      </c>
-      <c r="E12" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="F12" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="G12" s="1"/>
-    </row>
-    <row r="13" spans="1:29" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B13" s="3" t="s">
+      <c r="B12" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D12" s="28"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="17"/>
+    </row>
+    <row r="13" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="D13" s="28" t="s">
-        <v>6</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="F13" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="G13" s="1"/>
-      <c r="J13" s="25"/>
-      <c r="L13" s="25"/>
-    </row>
-    <row r="14" spans="1:29" ht="60" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
-        <v>39</v>
+      <c r="B13" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D13" s="28"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="17"/>
+    </row>
+    <row r="14" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
+        <v>32</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="D14" s="29" t="s">
-        <v>9</v>
-      </c>
-      <c r="E14" s="14" t="s">
+      <c r="D14" s="28"/>
+      <c r="E14" s="13"/>
+      <c r="F14" s="17"/>
+    </row>
+    <row r="15" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" s="28"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="17"/>
+    </row>
+    <row r="16" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="D16" s="28"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="17"/>
+    </row>
+    <row r="17" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="E17" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="F14" s="18" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="15" spans="1:29" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>48</v>
-      </c>
-      <c r="D15" s="29" t="s">
-        <v>6</v>
-      </c>
-      <c r="E15" s="14" t="s">
-        <v>11</v>
-      </c>
-      <c r="F15" s="18" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="16" spans="1:29" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" s="12" t="s">
+      <c r="F17" s="19" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="20" t="s">
+      <c r="B18" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="D16" s="30" t="s">
-        <v>38</v>
-      </c>
-      <c r="E16" s="16" t="s">
+      <c r="D18" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="F16" s="20" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="C17" s="20" t="s">
-        <v>28</v>
-      </c>
-      <c r="D17" s="30" t="s">
-        <v>38</v>
-      </c>
-      <c r="E17" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="F17" s="20" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A18" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="C18" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="D18" s="30" t="s">
-        <v>38</v>
-      </c>
-      <c r="E18" s="16" t="s">
+      <c r="F18" s="19" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+      <c r="A19" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="D19" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="E19" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="F18" s="20" t="s">
-        <v>61</v>
+      <c r="F19" s="19" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G13"/>
+  <autoFilter ref="A1:G9"/>
   <sortState ref="AB3:AB8">
     <sortCondition ref="AB3"/>
   </sortState>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E18">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E19">
       <formula1>$AC$3:$AC$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D18">
-      <formula1>$AB$3:$AB$9</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D19">
+      <formula1>$AB$3:$AB$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
item cubo compras da operação portuárias
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="59">
   <si>
     <t>projeto</t>
   </si>
@@ -195,6 +195,15 @@
   </si>
   <si>
     <t>Painel DRE entregue, e utilizado em reunião de diretoria referente a maio 2023. Tratar a característica ambígua credora e devedora da conta 331803, para que exiba valor positivo ou negativo quando pertinente.</t>
+  </si>
+  <si>
+    <t>Criar cubo dos itens de compras nas OS, para comparação com cubo de compras</t>
+  </si>
+  <si>
+    <t>por iniciar</t>
+  </si>
+  <si>
+    <t>Itens de OS de tipos 5 e 11 são comparados com o cubo de pedido de compra, mas o vínculo não é correto, pois os itens da OS são produtos e os itens do log de custo são números de NF.</t>
   </si>
 </sst>
 </file>
@@ -899,7 +908,9 @@
         <v>49</v>
       </c>
       <c r="G7" s="1"/>
-      <c r="AB7" s="5"/>
+      <c r="AB7" s="5" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="8" spans="1:29" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
@@ -957,7 +968,7 @@
         <v>34</v>
       </c>
       <c r="D10" s="28" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="E10" s="13" t="s">
         <v>12</v>
@@ -994,64 +1005,62 @@
         <v>40</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>41</v>
-      </c>
-      <c r="D12" s="28"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="17"/>
-    </row>
-    <row r="13" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+      <c r="D12" s="28" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="13" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>32</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="17" t="s">
-        <v>41</v>
-      </c>
+      <c r="C13" s="17"/>
       <c r="D13" s="28"/>
       <c r="E13" s="13"/>
       <c r="F13" s="17"/>
     </row>
-    <row r="14" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>32</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="17" t="s">
-        <v>41</v>
-      </c>
+      <c r="C14" s="17"/>
       <c r="D14" s="28"/>
       <c r="E14" s="13"/>
       <c r="F14" s="17"/>
     </row>
-    <row r="15" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>32</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="17" t="s">
-        <v>41</v>
-      </c>
+      <c r="C15" s="17"/>
       <c r="D15" s="28"/>
       <c r="E15" s="13"/>
       <c r="F15" s="17"/>
     </row>
-    <row r="16" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>32</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="17" t="s">
-        <v>41</v>
-      </c>
+      <c r="C16" s="17"/>
       <c r="D16" s="28"/>
       <c r="E16" s="13"/>
       <c r="F16" s="17"/>
@@ -1126,7 +1135,7 @@
       <formula1>$AC$3:$AC$5</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D19">
-      <formula1>$AB$3:$AB$6</formula1>
+      <formula1>$AB$3:$AB$7</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
atualizações do projeto de desempenho das operações portuárias
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="65">
   <si>
     <t>projeto</t>
   </si>
@@ -204,6 +204,24 @@
   </si>
   <si>
     <t>Itens de OS de tipos 5 e 11 são comparados com o cubo de pedido de compra, mas o vínculo não é correto, pois os itens da OS são produtos e os itens do log de custo são números de NF.</t>
+  </si>
+  <si>
+    <t>Criar relatório de provisões para confronto com valor do log de custo</t>
+  </si>
+  <si>
+    <t>Após orientação do Rodrigo sobre o funcionamento da tabela SRT, devo alterar o cubo de provisões para criar um campo do valor "gerencial" provisionado por mês</t>
+  </si>
+  <si>
+    <t>Adaptar cubo de log de custos para trazer o valor de provisões</t>
+  </si>
+  <si>
+    <t>Encontrado o valor mensal de provisão, criar um campo na consulta de log para que se compare o valor provisionado com o valor atribuído às OS portuárias</t>
+  </si>
+  <si>
+    <t>Verificar correção dos itens duplicados nas OS</t>
+  </si>
+  <si>
+    <t>Entender por qual motivo as exclusões realizadas pela Marília de apontamentos repetidos em OS não são encontrados pelo Paulo.</t>
   </si>
 </sst>
 </file>
@@ -717,7 +735,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AC19"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" customWidth="1"/>
@@ -733,7 +751,7 @@
     <col min="28" max="28" width="25.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="18.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -756,7 +774,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
@@ -776,14 +794,8 @@
         <v>55</v>
       </c>
       <c r="G2" s="1"/>
-      <c r="AB2" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="AC2" s="5" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:29" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:12" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
         <v>2</v>
       </c>
@@ -803,14 +815,8 @@
         <v>45</v>
       </c>
       <c r="G3" s="1"/>
-      <c r="AB3" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC3" s="5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:29" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:12" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>2</v>
       </c>
@@ -830,14 +836,8 @@
         <v>47</v>
       </c>
       <c r="G4" s="1"/>
-      <c r="AB4" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="AC4" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:29" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:12" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="20" t="s">
         <v>2</v>
       </c>
@@ -857,14 +857,8 @@
         <v>46</v>
       </c>
       <c r="G5" s="1"/>
-      <c r="AB5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="AC5" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:29" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
         <v>2</v>
       </c>
@@ -884,11 +878,8 @@
         <v>37</v>
       </c>
       <c r="G6" s="1"/>
-      <c r="AB6" s="5" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:29" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:12" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>3</v>
       </c>
@@ -908,11 +899,8 @@
         <v>49</v>
       </c>
       <c r="G7" s="1"/>
-      <c r="AB7" s="5" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="1:29" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:12" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>3</v>
       </c>
@@ -932,9 +920,8 @@
         <v>42</v>
       </c>
       <c r="G8" s="1"/>
-      <c r="AB8" s="5"/>
-    </row>
-    <row r="9" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>3</v>
       </c>
@@ -957,7 +944,7 @@
       <c r="J9" s="24"/>
       <c r="L9" s="24"/>
     </row>
-    <row r="10" spans="1:29" ht="60" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>32</v>
       </c>
@@ -977,7 +964,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="11" spans="1:29" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>32</v>
       </c>
@@ -997,7 +984,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:29" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>32</v>
       </c>
@@ -1017,63 +1004,95 @@
         <v>58</v>
       </c>
     </row>
-    <row r="13" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>32</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="28"/>
-      <c r="E13" s="13"/>
-      <c r="F13" s="17"/>
-    </row>
-    <row r="14" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C13" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>32</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="17"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="13"/>
-      <c r="F14" s="17"/>
-    </row>
-    <row r="15" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C14" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="D14" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>32</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C15" s="17"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="17"/>
-    </row>
-    <row r="16" spans="1:29" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="17"/>
-      <c r="D16" s="28"/>
-      <c r="E16" s="13"/>
-      <c r="F16" s="17"/>
-    </row>
-    <row r="17" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C15" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="D15" s="28" t="s">
+        <v>57</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>19</v>
+      </c>
+      <c r="D16" s="29" t="s">
+        <v>31</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="19" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="C17" s="19" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D17" s="29" t="s">
         <v>31</v>
@@ -1082,60 +1101,85 @@
         <v>12</v>
       </c>
       <c r="F17" s="19" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="C18" s="19" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="D18" s="29" t="s">
         <v>31</v>
       </c>
       <c r="E18" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="F18" s="19" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A42" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A44" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B44" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F18" s="19" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A19" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="D19" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="E19" s="15" t="s">
-        <v>13</v>
-      </c>
-      <c r="F19" s="19" t="s">
-        <v>50</v>
-      </c>
+    </row>
+    <row r="45" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A45" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A46" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A47" s="5"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G9"/>
-  <sortState ref="AB3:AB8">
-    <sortCondition ref="AB3"/>
+  <sortState ref="A43:A48">
+    <sortCondition ref="A3"/>
   </sortState>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E19">
-      <formula1>$AC$3:$AC$5</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E2:E18">
+      <formula1>$B$42:$B$44</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D19">
-      <formula1>$AB$3:$AB$7</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D18">
+      <formula1>$A$42:$A$46</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
alteração de status dos demais projetos
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -785,7 +785,7 @@
         <v>20</v>
       </c>
       <c r="D2" s="25" t="s">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="E2" s="12" t="s">
         <v>11</v>
@@ -890,7 +890,7 @@
         <v>15</v>
       </c>
       <c r="D7" s="27" t="s">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>11</v>
@@ -932,7 +932,7 @@
         <v>36</v>
       </c>
       <c r="D9" s="27" t="s">
-        <v>6</v>
+        <v>31</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
atualização de status do cubo de provisões da folha
</commit_message>
<xml_diff>
--- a/projetos.xlsx
+++ b/projetos.xlsx
@@ -15,7 +15,7 @@
     <sheet name="status" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">status!$A$1:$G$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">status!$A$1:$G$18</definedName>
   </definedNames>
   <calcPr calcId="152511"/>
   <extLst>
@@ -1015,7 +1015,7 @@
         <v>59</v>
       </c>
       <c r="D13" s="28" t="s">
-        <v>57</v>
+        <v>9</v>
       </c>
       <c r="E13" s="13" t="s">
         <v>11</v>
@@ -1035,7 +1035,7 @@
         <v>61</v>
       </c>
       <c r="D14" s="28" t="s">
-        <v>57</v>
+        <v>9</v>
       </c>
       <c r="E14" s="13" t="s">
         <v>11</v>
@@ -1055,7 +1055,7 @@
         <v>63</v>
       </c>
       <c r="D15" s="28" t="s">
-        <v>57</v>
+        <v>9</v>
       </c>
       <c r="E15" s="13" t="s">
         <v>11</v>
@@ -1170,7 +1170,7 @@
       <c r="A47" s="5"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G9"/>
+  <autoFilter ref="A1:G18"/>
   <sortState ref="A43:A48">
     <sortCondition ref="A3"/>
   </sortState>

</xml_diff>